<commit_message>
removed MGS diagnosis, added event study diagnosis & data reconstruction
</commit_message>
<xml_diff>
--- a/output/MONTHLY_MASTER.xlsx
+++ b/output/MONTHLY_MASTER.xlsx
@@ -576,20 +576,20 @@
         <v>3.8</v>
       </c>
       <c r="M2" t="n">
-        <v>98.37435241312053</v>
+        <v>98.37437931413426</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>102.9251333120346</v>
+        <v>102.9251279614441</v>
       </c>
       <c r="P2" t="n">
-        <v>119.1508655070364</v>
+        <v>119.1508424775353</v>
       </c>
       <c r="Q2" t="n">
-        <v>99.65450957691874</v>
+        <v>99.65451082203609</v>
       </c>
       <c r="R2" t="n">
-        <v>107.2503476708191</v>
+        <v>107.2503638772904</v>
       </c>
     </row>
     <row r="3">
@@ -628,20 +628,20 @@
         <v>3.87</v>
       </c>
       <c r="M3" t="n">
-        <v>103.7854324264138</v>
+        <v>103.7854391426815</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>105.9545259663922</v>
+        <v>105.954536906119</v>
       </c>
       <c r="P3" t="n">
-        <v>136.3440409828611</v>
+        <v>136.3440312416755</v>
       </c>
       <c r="Q3" t="n">
-        <v>107.1575164598785</v>
+        <v>107.1575374224943</v>
       </c>
       <c r="R3" t="n">
-        <v>114.8381568713302</v>
+        <v>114.8381367412892</v>
       </c>
     </row>
     <row r="4">
@@ -680,20 +680,20 @@
         <v>3.9</v>
       </c>
       <c r="M4" t="n">
-        <v>107.2268981995812</v>
+        <v>107.226925403209</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>104.51198238802</v>
+        <v>104.511984051493</v>
       </c>
       <c r="P4" t="n">
-        <v>138.4846910741614</v>
+        <v>138.4846701505982</v>
       </c>
       <c r="Q4" t="n">
-        <v>110.2193209114166</v>
+        <v>110.2193255798025</v>
       </c>
       <c r="R4" t="n">
-        <v>125.4287381519302</v>
+        <v>125.4287391227943</v>
       </c>
     </row>
     <row r="5">
@@ -732,20 +732,20 @@
         <v>3.85</v>
       </c>
       <c r="M5" t="n">
-        <v>107.2986685583297</v>
+        <v>107.2986638955405</v>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
-        <v>109.060228241279</v>
+        <v>109.060232891112</v>
       </c>
       <c r="P5" t="n">
-        <v>161.8369482853855</v>
+        <v>161.8369129508672</v>
       </c>
       <c r="Q5" t="n">
-        <v>113.8251468684475</v>
+        <v>113.8251771247492</v>
       </c>
       <c r="R5" t="n">
-        <v>117.5917170424015</v>
+        <v>117.5917032501909</v>
       </c>
     </row>
     <row r="6">
@@ -784,20 +784,20 @@
         <v>3.91</v>
       </c>
       <c r="M6" t="n">
-        <v>103.4372897718519</v>
+        <v>103.4372831158966</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
-        <v>107.1257172336449</v>
+        <v>107.125732424712</v>
       </c>
       <c r="P6" t="n">
-        <v>162.8126727881289</v>
+        <v>162.8126713659201</v>
       </c>
       <c r="Q6" t="n">
-        <v>112.8121562901202</v>
+        <v>112.8121785107685</v>
       </c>
       <c r="R6" t="n">
-        <v>111.7934227359978</v>
+        <v>111.7934173314091</v>
       </c>
     </row>
     <row r="7">
@@ -836,20 +836,20 @@
         <v>4.01</v>
       </c>
       <c r="M7" t="n">
-        <v>103.090531340004</v>
+        <v>103.0905340395417</v>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
-        <v>104.4556673562581</v>
+        <v>104.455681961217</v>
       </c>
       <c r="P7" t="n">
-        <v>158.8971828779311</v>
+        <v>158.8971904713783</v>
       </c>
       <c r="Q7" t="n">
-        <v>113.3859446803167</v>
+        <v>113.3859757294869</v>
       </c>
       <c r="R7" t="n">
-        <v>124.5922702309507</v>
+        <v>124.5922544857025</v>
       </c>
     </row>
     <row r="8">
@@ -888,20 +888,20 @@
         <v>4.06</v>
       </c>
       <c r="M8" t="n">
-        <v>103.302176021462</v>
+        <v>103.3021835889733</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
-        <v>106.1342529599382</v>
+        <v>106.1342394942913</v>
       </c>
       <c r="P8" t="n">
-        <v>165.1331929909585</v>
+        <v>165.1331684714696</v>
       </c>
       <c r="Q8" t="n">
-        <v>116.3730983436907</v>
+        <v>116.373107217383</v>
       </c>
       <c r="R8" t="n">
-        <v>130.0499230408035</v>
+        <v>130.0499070101017</v>
       </c>
     </row>
     <row r="9">
@@ -940,20 +940,20 @@
         <v>4.39</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>97.91436790685036</v>
+        <v>97.91435587116247</v>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" s="3" t="n">
-        <v>103.7373899586908</v>
+        <v>103.7373735524711</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>126.3458683842429</v>
+        <v>126.3458502016431</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>114.2937057901785</v>
+        <v>114.2937142177215</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>110.8244327959167</v>
+        <v>110.8244580267431</v>
       </c>
     </row>
     <row r="10">
@@ -992,20 +992,20 @@
         <v>4.14</v>
       </c>
       <c r="M10" t="n">
-        <v>92.99771169562935</v>
+        <v>92.99771568067506</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
-        <v>104.3622873883022</v>
+        <v>104.3622869190377</v>
       </c>
       <c r="P10" t="n">
-        <v>132.009839613264</v>
+        <v>132.0098264396057</v>
       </c>
       <c r="Q10" t="n">
-        <v>117.0920419668925</v>
+        <v>117.0920554929684</v>
       </c>
       <c r="R10" t="n">
-        <v>124.9086172806174</v>
+        <v>124.9086175343668</v>
       </c>
     </row>
     <row r="11">
@@ -1044,20 +1044,20 @@
         <v>4.37</v>
       </c>
       <c r="M11" t="n">
-        <v>94.8549486543678</v>
+        <v>94.85494357025031</v>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="n">
-        <v>105.9863722317266</v>
+        <v>105.9863903690044</v>
       </c>
       <c r="P11" t="n">
-        <v>156.4566706218505</v>
+        <v>156.4566163442289</v>
       </c>
       <c r="Q11" t="n">
-        <v>121.5180672495698</v>
+        <v>121.5180934038163</v>
       </c>
       <c r="R11" t="n">
-        <v>144.3417347405544</v>
+        <v>144.3417358255002</v>
       </c>
     </row>
     <row r="12">
@@ -1096,20 +1096,20 @@
         <v>4.2</v>
       </c>
       <c r="M12" t="n">
-        <v>94.86997350499934</v>
+        <v>94.86998331538972</v>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="n">
-        <v>104.3279079420143</v>
+        <v>104.3278962000952</v>
       </c>
       <c r="P12" t="n">
-        <v>167.3821823018771</v>
+        <v>167.382138110253</v>
       </c>
       <c r="Q12" t="n">
-        <v>128.9172226968794</v>
+        <v>128.9172388212942</v>
       </c>
       <c r="R12" t="n">
-        <v>138.5044373696624</v>
+        <v>138.5044698082455</v>
       </c>
     </row>
     <row r="13">
@@ -1148,20 +1148,20 @@
         <v>4.19</v>
       </c>
       <c r="M13" t="n">
-        <v>95.71995150182654</v>
+        <v>95.71995413971702</v>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
-        <v>104.8390101873304</v>
+        <v>104.8389793997337</v>
       </c>
       <c r="P13" t="n">
-        <v>169.5993971284184</v>
+        <v>169.5993967191258</v>
       </c>
       <c r="Q13" t="n">
-        <v>131.6284315770084</v>
+        <v>131.6284254882268</v>
       </c>
       <c r="R13" t="n">
-        <v>165.2180509659574</v>
+        <v>165.2180686480234</v>
       </c>
     </row>
     <row r="14">
@@ -1200,20 +1200,20 @@
         <v>3.85</v>
       </c>
       <c r="M14" t="n">
-        <v>93.39149222643324</v>
+        <v>93.39149017090939</v>
       </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
-        <v>107.4252560185794</v>
+        <v>107.4252340663844</v>
       </c>
       <c r="P14" t="n">
-        <v>157.850361035621</v>
+        <v>157.8503590096901</v>
       </c>
       <c r="Q14" t="n">
-        <v>132.8506140840422</v>
+        <v>132.8506279205694</v>
       </c>
       <c r="R14" t="n">
-        <v>140.2861991479637</v>
+        <v>140.2861989370778</v>
       </c>
     </row>
     <row r="15">
@@ -1252,20 +1252,20 @@
         <v>3.92</v>
       </c>
       <c r="M15" t="n">
-        <v>96.61515540722515</v>
+        <v>96.61513818935046</v>
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
-        <v>112.9983532657839</v>
+        <v>112.9983331891411</v>
       </c>
       <c r="P15" t="n">
-        <v>156.9901673184638</v>
+        <v>156.9901723540284</v>
       </c>
       <c r="Q15" t="n">
-        <v>127.1420315915643</v>
+        <v>127.1420532726359</v>
       </c>
       <c r="R15" t="n">
-        <v>153.1695141132298</v>
+        <v>153.1695165286483</v>
       </c>
     </row>
     <row r="16">
@@ -1304,20 +1304,20 @@
         <v>3.78</v>
       </c>
       <c r="M16" t="n">
-        <v>102.2242743408087</v>
+        <v>102.2242608983033</v>
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
-        <v>114.4279308201674</v>
+        <v>114.4279145234736</v>
       </c>
       <c r="P16" t="n">
-        <v>161.9969147950128</v>
+        <v>161.9968974500579</v>
       </c>
       <c r="Q16" t="n">
-        <v>127.0998681507231</v>
+        <v>127.0998935232199</v>
       </c>
       <c r="R16" t="n">
-        <v>163.311454393376</v>
+        <v>163.3114747181821</v>
       </c>
     </row>
     <row r="17">
@@ -1356,20 +1356,20 @@
         <v>3.88</v>
       </c>
       <c r="M17" t="n">
-        <v>100.5136855613799</v>
+        <v>100.5136933412754</v>
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
-        <v>114.7334971738379</v>
+        <v>114.7334716499635</v>
       </c>
       <c r="P17" t="n">
-        <v>151.2208082314584</v>
+        <v>151.2207662996651</v>
       </c>
       <c r="Q17" t="n">
-        <v>126.6434746625855</v>
+        <v>126.6435094879424</v>
       </c>
       <c r="R17" t="n">
-        <v>170.9932868619028</v>
+        <v>170.9933243162914</v>
       </c>
     </row>
     <row r="18">
@@ -1408,20 +1408,20 @@
         <v>3.92</v>
       </c>
       <c r="M18" t="n">
-        <v>97.44518759706334</v>
+        <v>97.44517673643821</v>
       </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
-        <v>118.6449004588067</v>
+        <v>118.6448871132939</v>
       </c>
       <c r="P18" t="n">
-        <v>154.6324050847008</v>
+        <v>154.6323523027171</v>
       </c>
       <c r="Q18" t="n">
-        <v>125.0320521036864</v>
+        <v>125.0320445626484</v>
       </c>
       <c r="R18" t="n">
-        <v>175.0948719598003</v>
+        <v>175.0948947813557</v>
       </c>
     </row>
     <row r="19">
@@ -1460,20 +1460,20 @@
         <v>3.75</v>
       </c>
       <c r="M19" t="n">
-        <v>97.66721710798907</v>
+        <v>97.66720564302037</v>
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
-        <v>120.4485781255417</v>
+        <v>120.4485506971055</v>
       </c>
       <c r="P19" t="n">
-        <v>149.5178493730118</v>
+        <v>149.5178272930565</v>
       </c>
       <c r="Q19" t="n">
-        <v>125.8710784560445</v>
+        <v>125.8710954805805</v>
       </c>
       <c r="R19" t="n">
-        <v>187.2039845143634</v>
+        <v>187.203999313535</v>
       </c>
     </row>
     <row r="20">
@@ -1512,20 +1512,20 @@
         <v>3.6</v>
       </c>
       <c r="M20" t="n">
-        <v>97.4801909159526</v>
+        <v>97.48019946771805</v>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
-        <v>121.6363885335569</v>
+        <v>121.6363789522458</v>
       </c>
       <c r="P20" t="n">
-        <v>160.3382065564388</v>
+        <v>160.3381463174803</v>
       </c>
       <c r="Q20" t="n">
-        <v>125.6392392447484</v>
+        <v>125.6392337727614</v>
       </c>
       <c r="R20" t="n">
-        <v>192.6505024756831</v>
+        <v>192.6504523376468</v>
       </c>
     </row>
     <row r="21">
@@ -1564,20 +1564,20 @@
         <v>3.59</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>101.6910556253835</v>
+        <v>101.6910734545936</v>
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" s="3" t="n">
-        <v>125.5703290778238</v>
+        <v>125.5703067507107</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>160.8174633718208</v>
+        <v>160.8174303405723</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>127.4272803482186</v>
+        <v>127.4272951004723</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>192.8311702729623</v>
+        <v>192.8311927259122</v>
       </c>
     </row>
     <row r="22">
@@ -1616,20 +1616,20 @@
         <v>3.55</v>
       </c>
       <c r="M22" t="n">
-        <v>100.8279050240244</v>
+        <v>100.8278962686602</v>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
-        <v>125.1852186716605</v>
+        <v>125.1851818176587</v>
       </c>
       <c r="P22" t="n">
-        <v>160.9423260976588</v>
+        <v>160.9422938150745</v>
       </c>
       <c r="Q22" t="n">
-        <v>127.0650836530197</v>
+        <v>127.0651196412199</v>
       </c>
       <c r="R22" t="n">
-        <v>214.4158989623239</v>
+        <v>214.4159669650777</v>
       </c>
     </row>
     <row r="23">
@@ -1668,20 +1668,20 @@
         <v>3.61</v>
       </c>
       <c r="M23" t="n">
-        <v>104.9686530019274</v>
+        <v>104.9686623549289</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
-        <v>128.855121543894</v>
+        <v>128.8550971279553</v>
       </c>
       <c r="P23" t="n">
-        <v>161.2025976966638</v>
+        <v>161.2025570058669</v>
       </c>
       <c r="Q23" t="n">
-        <v>129.3323231424372</v>
+        <v>129.3323213114286</v>
       </c>
       <c r="R23" t="n">
-        <v>213.1240928880147</v>
+        <v>213.1240957193673</v>
       </c>
     </row>
     <row r="24">
@@ -1720,20 +1720,20 @@
         <v>4.35</v>
       </c>
       <c r="M24" t="n">
-        <v>100.6919032797179</v>
+        <v>100.6919068134812</v>
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="n">
-        <v>124.1260092071735</v>
+        <v>124.1259821643854</v>
       </c>
       <c r="P24" t="n">
-        <v>161.425674016797</v>
+        <v>161.4256676533209</v>
       </c>
       <c r="Q24" t="n">
-        <v>126.193016567386</v>
+        <v>126.1930389152258</v>
       </c>
       <c r="R24" t="n">
-        <v>229.9730049430111</v>
+        <v>229.9729868103053</v>
       </c>
     </row>
     <row r="25">
@@ -1772,20 +1772,20 @@
         <v>4.22</v>
       </c>
       <c r="M25" t="n">
-        <v>102.3427116603758</v>
+        <v>102.3427256635119</v>
       </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="n">
-        <v>128.142287604888</v>
+        <v>128.1422681035399</v>
       </c>
       <c r="P25" t="n">
-        <v>170.9328046579934</v>
+        <v>170.9327775709012</v>
       </c>
       <c r="Q25" t="n">
-        <v>129.2578825667346</v>
+        <v>129.2579059594954</v>
       </c>
       <c r="R25" t="n">
-        <v>226.0251473102865</v>
+        <v>226.0250818909762</v>
       </c>
     </row>
     <row r="26">
@@ -1824,20 +1824,20 @@
         <v>4.14</v>
       </c>
       <c r="M26" t="n">
-        <v>106.5026944496907</v>
+        <v>106.5027111391762</v>
       </c>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
-        <v>131.7046669808429</v>
+        <v>131.7046784205591</v>
       </c>
       <c r="P26" t="n">
-        <v>180.2204923419858</v>
+        <v>180.2204869209639</v>
       </c>
       <c r="Q26" t="n">
-        <v>128.8888500812333</v>
+        <v>128.888862843853</v>
       </c>
       <c r="R26" t="n">
-        <v>255.4749715774079</v>
+        <v>255.4749771464934</v>
       </c>
     </row>
     <row r="27">
@@ -1876,20 +1876,20 @@
         <v>4.04</v>
       </c>
       <c r="M27" t="n">
-        <v>108.4766364113775</v>
+        <v>108.4766487885541</v>
       </c>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
-        <v>127.5850664677137</v>
+        <v>127.5850532859377</v>
       </c>
       <c r="P27" t="n">
-        <v>201.5676005619055</v>
+        <v>201.5675636521823</v>
       </c>
       <c r="Q27" t="n">
-        <v>129.5697670344082</v>
+        <v>129.56975613149</v>
       </c>
       <c r="R27" t="n">
-        <v>276.8609850423358</v>
+        <v>276.8609457962618</v>
       </c>
     </row>
     <row r="28">
@@ -1928,20 +1928,20 @@
         <v>4.13</v>
       </c>
       <c r="M28" t="n">
-        <v>114.8296224671624</v>
+        <v>114.8296474163053</v>
       </c>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="n">
-        <v>129.6918335723266</v>
+        <v>129.691815794948</v>
       </c>
       <c r="P28" t="n">
-        <v>225.6404345775087</v>
+        <v>225.640427704635</v>
       </c>
       <c r="Q28" t="n">
-        <v>132.4758718770172</v>
+        <v>132.4758762230286</v>
       </c>
       <c r="R28" t="n">
-        <v>284.1496838719969</v>
+        <v>284.149719070278</v>
       </c>
     </row>
     <row r="29">
@@ -1980,20 +1980,20 @@
         <v>4.05</v>
       </c>
       <c r="M29" t="n">
-        <v>118.927021139412</v>
+        <v>118.9270270997291</v>
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
-        <v>128.9233721881446</v>
+        <v>128.9233657163314</v>
       </c>
       <c r="P29" t="n">
-        <v>245.5288386826826</v>
+        <v>245.5288108796182</v>
       </c>
       <c r="Q29" t="n">
-        <v>127.4250864497548</v>
+        <v>127.4250985099636</v>
       </c>
       <c r="R29" t="n">
-        <v>288.1720141601268</v>
+        <v>288.1719988319765</v>
       </c>
     </row>
     <row r="30">
@@ -2032,20 +2032,20 @@
         <v>3.87</v>
       </c>
       <c r="M30" t="n">
-        <v>123.9146663358798</v>
+        <v>123.9146732693287</v>
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="n">
-        <v>128.8062469751864</v>
+        <v>128.8062361863109</v>
       </c>
       <c r="P30" t="n">
-        <v>262.69340801526</v>
+        <v>262.6933750264289</v>
       </c>
       <c r="Q30" t="n">
-        <v>129.4759106555026</v>
+        <v>129.4759109458239</v>
       </c>
       <c r="R30" t="n">
-        <v>290.8279023292222</v>
+        <v>290.8279314111676</v>
       </c>
     </row>
     <row r="31">
@@ -2084,20 +2084,20 @@
         <v>3.91</v>
       </c>
       <c r="M31" t="n">
-        <v>126.4622093578761</v>
+        <v>126.462218589772</v>
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="n">
-        <v>134.3879684085865</v>
+        <v>134.3879958063733</v>
       </c>
       <c r="P31" t="n">
-        <v>299.5791662589999</v>
+        <v>299.5791223136418</v>
       </c>
       <c r="Q31" t="n">
-        <v>127.2420651987168</v>
+        <v>127.2420794613961</v>
       </c>
       <c r="R31" t="n">
-        <v>310.6826702694797</v>
+        <v>310.6827126233402</v>
       </c>
     </row>
     <row r="32">
@@ -2136,20 +2136,20 @@
         <v>3.99</v>
       </c>
       <c r="M32" t="n">
-        <v>125.829028678091</v>
+        <v>125.8290543566511</v>
       </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="n">
-        <v>130.6499932481345</v>
+        <v>130.6500040611811</v>
       </c>
       <c r="P32" t="n">
-        <v>358.4797240419714</v>
+        <v>358.4796900554085</v>
       </c>
       <c r="Q32" t="n">
-        <v>126.2873096805411</v>
+        <v>126.287305970308</v>
       </c>
       <c r="R32" t="n">
-        <v>321.9736316093327</v>
+        <v>321.9735860178054</v>
       </c>
     </row>
     <row r="33">
@@ -2188,20 +2188,20 @@
         <v>3.89</v>
       </c>
       <c r="M33" t="n">
-        <v>130.0740281802776</v>
+        <v>130.0740409323505</v>
       </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="n">
-        <v>132.3059087660324</v>
+        <v>132.3059241268977</v>
       </c>
       <c r="P33" t="n">
-        <v>351.2770725678774</v>
+        <v>351.2770813795991</v>
       </c>
       <c r="Q33" t="n">
-        <v>128.9823706860797</v>
+        <v>128.9823608361818</v>
       </c>
       <c r="R33" t="n">
-        <v>358.6836158265253</v>
+        <v>358.6835802992477</v>
       </c>
     </row>
     <row r="34">
@@ -2240,20 +2240,20 @@
         <v>3.92</v>
       </c>
       <c r="M34" t="n">
-        <v>126.1729698308357</v>
+        <v>126.1729967345801</v>
       </c>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="n">
-        <v>134.9772047105333</v>
+        <v>134.9771887690834</v>
       </c>
       <c r="P34" t="n">
-        <v>364.56999731877</v>
+        <v>364.5699443217296</v>
       </c>
       <c r="Q34" t="n">
-        <v>128.7377192008835</v>
+        <v>128.7377194480933</v>
       </c>
       <c r="R34" t="n">
-        <v>365.8627718475248</v>
+        <v>365.8628096140748</v>
       </c>
     </row>
     <row r="35">
@@ -2292,20 +2292,20 @@
         <v>3.94</v>
       </c>
       <c r="M35" t="n">
-        <v>124.7592791128298</v>
+        <v>124.7592790972883</v>
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="n">
-        <v>132.4268417956351</v>
+        <v>132.4268077234238</v>
       </c>
       <c r="P35" t="n">
-        <v>407.2568242476109</v>
+        <v>407.2567016141663</v>
       </c>
       <c r="Q35" t="n">
-        <v>128.9862983543279</v>
+        <v>128.9863175629031</v>
       </c>
       <c r="R35" t="n">
-        <v>426.6522381284307</v>
+        <v>426.6522836175188</v>
       </c>
     </row>
     <row r="36">
@@ -2344,22 +2344,22 @@
         <v>3.89</v>
       </c>
       <c r="M36" t="n">
-        <v>123.0406191204165</v>
+        <v>123.0406248620192</v>
       </c>
       <c r="N36" t="n">
         <v>100</v>
       </c>
       <c r="O36" t="n">
-        <v>131.002967965358</v>
+        <v>131.0029557678561</v>
       </c>
       <c r="P36" t="n">
-        <v>428.741756020617</v>
+        <v>428.7416958643345</v>
       </c>
       <c r="Q36" t="n">
-        <v>125.3182064797862</v>
+        <v>125.3182235495241</v>
       </c>
       <c r="R36" t="n">
-        <v>475.2096719155409</v>
+        <v>475.209699853383</v>
       </c>
     </row>
     <row r="37">
@@ -2398,22 +2398,22 @@
         <v>3.91</v>
       </c>
       <c r="M37" t="n">
-        <v>130.6636172683421</v>
+        <v>130.6636113803382</v>
       </c>
       <c r="N37" t="n">
-        <v>107.9068535967807</v>
+        <v>107.9068716307397</v>
       </c>
       <c r="O37" t="n">
-        <v>146.1028239065589</v>
+        <v>146.102791550257</v>
       </c>
       <c r="P37" t="n">
-        <v>483.9690157749015</v>
+        <v>483.9688942647632</v>
       </c>
       <c r="Q37" t="n">
-        <v>131.2691748118108</v>
+        <v>131.2691768569645</v>
       </c>
       <c r="R37" t="n">
-        <v>529.0481624678202</v>
+        <v>529.0481313347783</v>
       </c>
     </row>
     <row r="38">
@@ -2452,22 +2452,22 @@
         <v>3.96</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>139.2056164180506</v>
+        <v>139.2056258832753</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>106.3691083949243</v>
+        <v>106.3691160582806</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>131.3476733803591</v>
+        <v>131.3476702181251</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>481.7522264914951</v>
+        <v>481.7521664380259</v>
       </c>
       <c r="Q38" s="3" t="n">
-        <v>135.6503149036956</v>
+        <v>135.6503322100426</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>594.7357518404923</v>
+        <v>594.7357546676351</v>
       </c>
     </row>
     <row r="39">
@@ -2506,22 +2506,22 @@
         <v>4.01</v>
       </c>
       <c r="M39" t="n">
-        <v>142.6418369256956</v>
+        <v>142.641849533851</v>
       </c>
       <c r="N39" t="n">
-        <v>105.1654984669877</v>
+        <v>105.1654995602039</v>
       </c>
       <c r="O39" t="n">
-        <v>131.4189668618227</v>
+        <v>131.418973283743</v>
       </c>
       <c r="P39" t="n">
-        <v>495.1229502711499</v>
+        <v>495.1228317869695</v>
       </c>
       <c r="Q39" t="n">
-        <v>137.0150992049531</v>
+        <v>137.0151291440982</v>
       </c>
       <c r="R39" t="n">
-        <v>610.1138713830129</v>
+        <v>610.1138568955213</v>
       </c>
     </row>
     <row r="40">
@@ -2560,22 +2560,22 @@
         <v>3.94</v>
       </c>
       <c r="M40" t="n">
-        <v>146.9024138460866</v>
+        <v>146.9023916097533</v>
       </c>
       <c r="N40" t="n">
-        <v>109.0363073319148</v>
+        <v>109.0363220291276</v>
       </c>
       <c r="O40" t="n">
-        <v>125.9932024296885</v>
+        <v>125.9931947422833</v>
       </c>
       <c r="P40" t="n">
-        <v>422.1024574773255</v>
+        <v>422.1023828395201</v>
       </c>
       <c r="Q40" t="n">
-        <v>139.2008118955735</v>
+        <v>139.2008112909151</v>
       </c>
       <c r="R40" t="n">
-        <v>526.8910107257163</v>
+        <v>526.8911074242171</v>
       </c>
     </row>
     <row r="41">
@@ -2614,22 +2614,22 @@
         <v>4.13</v>
       </c>
       <c r="M41" t="n">
-        <v>147.4340920994775</v>
+        <v>147.4341111277617</v>
       </c>
       <c r="N41" t="n">
-        <v>109.5091684597308</v>
+        <v>109.509164393151</v>
       </c>
       <c r="O41" t="n">
-        <v>130.9847594956829</v>
+        <v>130.9847637515667</v>
       </c>
       <c r="P41" t="n">
-        <v>404.2395951143506</v>
+        <v>404.239511451754</v>
       </c>
       <c r="Q41" t="n">
-        <v>144.1461671038865</v>
+        <v>144.1461535469353</v>
       </c>
       <c r="R41" t="n">
-        <v>556.1194588936313</v>
+        <v>556.1195037220255</v>
       </c>
     </row>
     <row r="42">
@@ -2668,22 +2668,22 @@
         <v>4.18</v>
       </c>
       <c r="M42" t="n">
-        <v>133.2035852260922</v>
+        <v>133.2035876385344</v>
       </c>
       <c r="N42" t="n">
-        <v>107.0029720569263</v>
+        <v>107.0029601689807</v>
       </c>
       <c r="O42" t="n">
-        <v>138.5566807474393</v>
+        <v>138.5566834795851</v>
       </c>
       <c r="P42" t="n">
-        <v>471.1892087500866</v>
+        <v>471.1891155701873</v>
       </c>
       <c r="Q42" t="n">
-        <v>136.4009904234624</v>
+        <v>136.400993784229</v>
       </c>
       <c r="R42" t="n">
-        <v>548.5945171348111</v>
+        <v>548.5944976602692</v>
       </c>
     </row>
     <row r="43">
@@ -2722,22 +2722,22 @@
         <v>4.2</v>
       </c>
       <c r="M43" t="n">
-        <v>127.5631042057019</v>
+        <v>127.5631139367955</v>
       </c>
       <c r="N43" t="n">
-        <v>104.2725520275478</v>
+        <v>104.2725472185836</v>
       </c>
       <c r="O43" t="n">
-        <v>142.833225335293</v>
+        <v>142.8332210981636</v>
       </c>
       <c r="P43" t="n">
-        <v>467.6745281688914</v>
+        <v>467.674440813632</v>
       </c>
       <c r="Q43" t="n">
-        <v>139.4605496607436</v>
+        <v>139.4605891434346</v>
       </c>
       <c r="R43" t="n">
-        <v>600.6630549006987</v>
+        <v>600.6631250671463</v>
       </c>
     </row>
     <row r="44">
@@ -2776,22 +2776,22 @@
         <v>4.07</v>
       </c>
       <c r="M44" t="n">
-        <v>135.7489377421829</v>
+        <v>135.7489273070298</v>
       </c>
       <c r="N44" t="n">
-        <v>105.4892597347121</v>
+        <v>105.4892771462662</v>
       </c>
       <c r="O44" t="n">
-        <v>140.9009984635527</v>
+        <v>140.9010087276071</v>
       </c>
       <c r="P44" t="n">
-        <v>548.3300286410381</v>
+        <v>548.3298859480752</v>
       </c>
       <c r="Q44" t="n">
-        <v>150.3657810341981</v>
+        <v>150.3657769395785</v>
       </c>
       <c r="R44" t="n">
-        <v>583.2115429774009</v>
+        <v>583.2114391753186</v>
       </c>
     </row>
     <row r="45">
@@ -2830,22 +2830,22 @@
         <v>4.04</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>140.3911295780967</v>
+        <v>140.3911412784824</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>105.3742421070274</v>
+        <v>105.3742580973803</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>141.4153006213441</v>
+        <v>141.4153239610622</v>
       </c>
       <c r="P45" s="3" t="n">
-        <v>662.7671940992731</v>
+        <v>662.7672123783553</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>154.9234408775778</v>
+        <v>154.9234639010021</v>
       </c>
       <c r="R45" s="3" t="n">
-        <v>625.4760372845677</v>
+        <v>625.4760446853923</v>
       </c>
     </row>
     <row r="46">
@@ -2884,22 +2884,22 @@
         <v>4.07</v>
       </c>
       <c r="M46" t="n">
-        <v>141.6206375231348</v>
+        <v>141.6206559267246</v>
       </c>
       <c r="N46" t="n">
-        <v>106.1477653572969</v>
+        <v>106.1477719305693</v>
       </c>
       <c r="O46" t="n">
-        <v>138.7948253799666</v>
+        <v>138.7948247229351</v>
       </c>
       <c r="P46" t="n">
-        <v>690.0455439308746</v>
+        <v>690.0454445362035</v>
       </c>
       <c r="Q46" t="n">
-        <v>153.4466175906661</v>
+        <v>153.446640483813</v>
       </c>
       <c r="R46" t="n">
-        <v>604.7793701667654</v>
+        <v>604.7793659445413</v>
       </c>
     </row>
     <row r="47">
@@ -2938,22 +2938,22 @@
         <v>4.08</v>
       </c>
       <c r="M47" t="n">
-        <v>137.2267386859551</v>
+        <v>137.2267381822569</v>
       </c>
       <c r="N47" t="n">
-        <v>105.5678559373695</v>
+        <v>105.5678698876209</v>
       </c>
       <c r="O47" t="n">
-        <v>138.8775199276695</v>
+        <v>138.8774963892861</v>
       </c>
       <c r="P47" t="n">
-        <v>619.5024510819627</v>
+        <v>619.5023778664427</v>
       </c>
       <c r="Q47" t="n">
-        <v>151.3406207237485</v>
+        <v>151.3406321520312</v>
       </c>
       <c r="R47" t="n">
-        <v>637.8591939297022</v>
+        <v>637.8592880561959</v>
       </c>
     </row>
     <row r="48">
@@ -2992,22 +2992,22 @@
         <v>4.12</v>
       </c>
       <c r="M48" t="n">
-        <v>137.6815139436231</v>
+        <v>137.6815078139948</v>
       </c>
       <c r="N48" t="n">
-        <v>99.27227076808762</v>
+        <v>99.27226917863887</v>
       </c>
       <c r="O48" t="n">
-        <v>140.7496584916715</v>
+        <v>140.7496698803698</v>
       </c>
       <c r="P48" t="n">
-        <v>573.8438203833832</v>
+        <v>573.8437759189012</v>
       </c>
       <c r="Q48" t="n">
-        <v>152.0282615147312</v>
+        <v>152.0282503484073</v>
       </c>
       <c r="R48" t="n">
-        <v>634.7137251446064</v>
+        <v>634.7136544366625</v>
       </c>
     </row>
     <row r="49">
@@ -3046,22 +3046,22 @@
         <v>4.07</v>
       </c>
       <c r="M49" t="n">
-        <v>137.5860030313972</v>
+        <v>137.5860085658455</v>
       </c>
       <c r="N49" t="n">
-        <v>102.6181026755944</v>
+        <v>102.6181129384897</v>
       </c>
       <c r="O49" t="n">
-        <v>143.5138046186817</v>
+        <v>143.5138086868331</v>
       </c>
       <c r="P49" t="n">
-        <v>518.7561987228327</v>
+        <v>518.7560983689061</v>
       </c>
       <c r="Q49" t="n">
-        <v>155.5198661230878</v>
+        <v>155.519890632612</v>
       </c>
       <c r="R49" t="n">
-        <v>621.9054997972504</v>
+        <v>621.905531508277</v>
       </c>
     </row>
     <row r="50">
@@ -3100,22 +3100,22 @@
         <v>4.06</v>
       </c>
       <c r="M50" t="n">
-        <v>137.1141146519014</v>
+        <v>137.1141189696269</v>
       </c>
       <c r="N50" t="n">
-        <v>107.0795765205354</v>
+        <v>107.0795842740744</v>
       </c>
       <c r="O50" t="n">
-        <v>146.3713786798411</v>
+        <v>146.3713810686816</v>
       </c>
       <c r="P50" t="n">
-        <v>565.6038414457677</v>
+        <v>565.6037016228415</v>
       </c>
       <c r="Q50" t="n">
-        <v>147.6605830250249</v>
+        <v>147.6605779565835</v>
       </c>
       <c r="R50" t="n">
-        <v>548.8876749810772</v>
+        <v>548.887844710132</v>
       </c>
     </row>
     <row r="51">
@@ -3156,22 +3156,22 @@
         <v>3.89</v>
       </c>
       <c r="M51" t="n">
-        <v>139.336016098401</v>
+        <v>139.3360225155159</v>
       </c>
       <c r="N51" t="n">
-        <v>105.8990978703931</v>
+        <v>105.8991047379914</v>
       </c>
       <c r="O51" t="n">
-        <v>147.8178109967531</v>
+        <v>147.8178262298555</v>
       </c>
       <c r="P51" t="n">
-        <v>604.9361540643881</v>
+        <v>604.9360435399484</v>
       </c>
       <c r="Q51" t="n">
-        <v>152.8088849608141</v>
+        <v>152.8088908346694</v>
       </c>
       <c r="R51" t="n">
-        <v>528.6764919306338</v>
+        <v>528.676572756164</v>
       </c>
     </row>
     <row r="52">
@@ -3212,22 +3212,22 @@
         <v>3.77</v>
       </c>
       <c r="M52" t="n">
-        <v>130.6616606042844</v>
+        <v>130.6616672049275</v>
       </c>
       <c r="N52" t="n">
-        <v>105.478670226392</v>
+        <v>105.4786772696969</v>
       </c>
       <c r="O52" t="n">
-        <v>151.5706880919802</v>
+        <v>151.57068519493</v>
       </c>
       <c r="P52" t="n">
-        <v>626.9116916366936</v>
+        <v>626.911656587465</v>
       </c>
       <c r="Q52" t="n">
-        <v>149.9793342422717</v>
+        <v>149.9793341718233</v>
       </c>
       <c r="R52" t="n">
-        <v>552.5542374534298</v>
+        <v>552.5542507675128</v>
       </c>
     </row>
     <row r="53">
@@ -3268,22 +3268,22 @@
         <v>3.79</v>
       </c>
       <c r="M53" t="n">
-        <v>130.3471179273247</v>
+        <v>130.3471148782864</v>
       </c>
       <c r="N53" t="n">
-        <v>106.7890706719482</v>
+        <v>106.7890682413534</v>
       </c>
       <c r="O53" t="n">
-        <v>153.3841037737506</v>
+        <v>153.3841248289915</v>
       </c>
       <c r="P53" t="n">
-        <v>725.9724894465655</v>
+        <v>725.9722932136233</v>
       </c>
       <c r="Q53" t="n">
-        <v>147.6443520180634</v>
+        <v>147.6443618362464</v>
       </c>
       <c r="R53" t="n">
-        <v>582.3533900285554</v>
+        <v>582.3535129129557</v>
       </c>
     </row>
     <row r="54">
@@ -3324,22 +3324,22 @@
         <v>3.78</v>
       </c>
       <c r="M54" t="n">
-        <v>132.9009840516329</v>
+        <v>132.9009821591039</v>
       </c>
       <c r="N54" t="n">
-        <v>101.951498264409</v>
+        <v>101.9515024236487</v>
       </c>
       <c r="O54" t="n">
-        <v>155.5749614035297</v>
+        <v>155.5749981614628</v>
       </c>
       <c r="P54" t="n">
-        <v>674.3004136992541</v>
+        <v>674.3002173821135</v>
       </c>
       <c r="Q54" t="n">
-        <v>146.9686700871717</v>
+        <v>146.9686785190884</v>
       </c>
       <c r="R54" t="n">
-        <v>576.4089002384981</v>
+        <v>576.4090809860535</v>
       </c>
     </row>
     <row r="55">
@@ -3380,22 +3380,22 @@
         <v>3.63</v>
       </c>
       <c r="M55" t="n">
-        <v>132.0036676533708</v>
+        <v>132.003676710339</v>
       </c>
       <c r="N55" t="n">
-        <v>103.109567990558</v>
+        <v>103.1095707351498</v>
       </c>
       <c r="O55" t="n">
-        <v>157.3957521180607</v>
+        <v>157.3957613876281</v>
       </c>
       <c r="P55" t="n">
-        <v>700.7811873826254</v>
+        <v>700.7810013622463</v>
       </c>
       <c r="Q55" t="n">
-        <v>146.7028029874216</v>
+        <v>146.7027954351074</v>
       </c>
       <c r="R55" t="n">
-        <v>564.3525845362965</v>
+        <v>564.3526509501054</v>
       </c>
     </row>
     <row r="56">
@@ -3436,22 +3436,22 @@
         <v>3.57</v>
       </c>
       <c r="M56" t="n">
-        <v>126.3233045360541</v>
+        <v>126.3232983855473</v>
       </c>
       <c r="N56" t="n">
-        <v>99.36476408527804</v>
+        <v>99.36477005460075</v>
       </c>
       <c r="O56" t="n">
-        <v>159.3202938113228</v>
+        <v>159.3202880687583</v>
       </c>
       <c r="P56" t="n">
-        <v>746.5165752644841</v>
+        <v>746.5164301582996</v>
       </c>
       <c r="Q56" t="n">
-        <v>134.2211227773932</v>
+        <v>134.2211395143011</v>
       </c>
       <c r="R56" t="n">
-        <v>554.2014193499281</v>
+        <v>554.2015674211221</v>
       </c>
     </row>
     <row r="57">
@@ -3492,22 +3492,22 @@
         <v>3.32</v>
       </c>
       <c r="M57" t="n">
-        <v>123.9468984536766</v>
+        <v>123.9469140318781</v>
       </c>
       <c r="N57" t="n">
-        <v>104.3048349383143</v>
+        <v>104.3048483124033</v>
       </c>
       <c r="O57" t="n">
-        <v>168.1140435107307</v>
+        <v>168.1140425045672</v>
       </c>
       <c r="P57" t="n">
-        <v>745.6465550333528</v>
+        <v>745.6463654752225</v>
       </c>
       <c r="Q57" t="n">
-        <v>130.4420373738354</v>
+        <v>130.4420535253333</v>
       </c>
       <c r="R57" t="n">
-        <v>590.0479861990748</v>
+        <v>590.0479468673916</v>
       </c>
     </row>
     <row r="58">
@@ -3548,22 +3548,22 @@
         <v>3.32</v>
       </c>
       <c r="M58" t="n">
-        <v>123.5424204929133</v>
+        <v>123.5424169180653</v>
       </c>
       <c r="N58" t="n">
-        <v>101.4397051339134</v>
+        <v>101.4397035575152</v>
       </c>
       <c r="O58" t="n">
-        <v>166.4830931447921</v>
+        <v>166.4830971312667</v>
       </c>
       <c r="P58" t="n">
-        <v>823.0183903742957</v>
+        <v>823.0182614392284</v>
       </c>
       <c r="Q58" t="n">
-        <v>137.3367221736694</v>
+        <v>137.3367261825612</v>
       </c>
       <c r="R58" t="n">
-        <v>562.584215808046</v>
+        <v>562.5843959169592</v>
       </c>
     </row>
     <row r="59">
@@ -3604,22 +3604,22 @@
         <v>3.41</v>
       </c>
       <c r="M59" t="n">
-        <v>127.4444859166779</v>
+        <v>127.4444897811629</v>
       </c>
       <c r="N59" t="n">
-        <v>100.2415046674174</v>
+        <v>100.2415208521123</v>
       </c>
       <c r="O59" t="n">
-        <v>159.2547222694569</v>
+        <v>159.2547206040478</v>
       </c>
       <c r="P59" t="n">
-        <v>885.15120713339</v>
+        <v>885.1510458637847</v>
       </c>
       <c r="Q59" t="n">
-        <v>137.6051346773174</v>
+        <v>137.6051098297774</v>
       </c>
       <c r="R59" t="n">
-        <v>556.3695463076609</v>
+        <v>556.3696984857902</v>
       </c>
     </row>
     <row r="60">
@@ -3660,22 +3660,22 @@
         <v>3.42</v>
       </c>
       <c r="M60" t="n">
-        <v>125.1405582976115</v>
+        <v>125.1405608042392</v>
       </c>
       <c r="N60" t="n">
-        <v>103.5306551242321</v>
+        <v>103.5306726769182</v>
       </c>
       <c r="O60" t="n">
-        <v>163.1831343307076</v>
+        <v>163.183138962069</v>
       </c>
       <c r="P60" t="n">
-        <v>874.3978439009703</v>
+        <v>874.3976718208912</v>
       </c>
       <c r="Q60" t="n">
-        <v>130.8143181597481</v>
+        <v>130.8143335801043</v>
       </c>
       <c r="R60" t="n">
-        <v>562.6970293463339</v>
+        <v>562.6970801657471</v>
       </c>
     </row>
     <row r="61">
@@ -3716,22 +3716,22 @@
         <v>3.3</v>
       </c>
       <c r="M61" t="n">
-        <v>125.087091146581</v>
+        <v>125.0871076727595</v>
       </c>
       <c r="N61" t="n">
-        <v>111.1020894514236</v>
+        <v>111.1020988385528</v>
       </c>
       <c r="O61" t="n">
-        <v>160.5442564974287</v>
+        <v>160.5442523433302</v>
       </c>
       <c r="P61" t="n">
-        <v>910.0527563558766</v>
+        <v>910.0524261324122</v>
       </c>
       <c r="Q61" t="n">
-        <v>137.1895770351216</v>
+        <v>137.1895719824042</v>
       </c>
       <c r="R61" t="n">
-        <v>575.6900688507883</v>
+        <v>575.6903160352576</v>
       </c>
     </row>
     <row r="62">
@@ -3772,22 +3772,22 @@
         <v>3.13</v>
       </c>
       <c r="M62" t="n">
-        <v>120.5205147296369</v>
+        <v>120.5205346117062</v>
       </c>
       <c r="N62" t="n">
-        <v>105.5018798846095</v>
+        <v>105.5018902039108</v>
       </c>
       <c r="O62" t="n">
-        <v>161.0046689266057</v>
+        <v>161.0046724724531</v>
       </c>
       <c r="P62" t="n">
-        <v>981.0313590388134</v>
+        <v>981.0311154115592</v>
       </c>
       <c r="Q62" t="n">
-        <v>126.3063635687722</v>
+        <v>126.3063643482481</v>
       </c>
       <c r="R62" t="n">
-        <v>660.2841369229099</v>
+        <v>660.2842564811732</v>
       </c>
     </row>
     <row r="63">
@@ -3828,22 +3828,22 @@
         <v>2.82</v>
       </c>
       <c r="M63" t="n">
-        <v>116.3340297358178</v>
+        <v>116.3340422430455</v>
       </c>
       <c r="N63" t="n">
-        <v>100.4157658322614</v>
+        <v>100.4157822537295</v>
       </c>
       <c r="O63" t="n">
-        <v>168.8879830510373</v>
+        <v>168.8879896166205</v>
       </c>
       <c r="P63" t="n">
-        <v>873.5949303866739</v>
+        <v>873.594741243671</v>
       </c>
       <c r="Q63" t="n">
-        <v>123.8707485504625</v>
+        <v>123.870733039185</v>
       </c>
       <c r="R63" t="n">
-        <v>634.469754989343</v>
+        <v>634.4697641616089</v>
       </c>
     </row>
     <row r="64">
@@ -3884,22 +3884,22 @@
         <v>3.35</v>
       </c>
       <c r="M64" t="n">
-        <v>100.9657909410796</v>
+        <v>100.9658004378637</v>
       </c>
       <c r="N64" t="n">
-        <v>98.15455245832322</v>
+        <v>98.15455206869096</v>
       </c>
       <c r="O64" t="n">
-        <v>146.6845799295042</v>
+        <v>146.6845856096126</v>
       </c>
       <c r="P64" t="n">
-        <v>753.0450754717348</v>
+        <v>753.0449321690423</v>
       </c>
       <c r="Q64" t="n">
-        <v>118.1931642685405</v>
+        <v>118.1931660495829</v>
       </c>
       <c r="R64" t="n">
-        <v>575.0329499182005</v>
+        <v>575.0330861557389</v>
       </c>
     </row>
     <row r="65">
@@ -3940,22 +3940,22 @@
         <v>2.89</v>
       </c>
       <c r="M65" t="n">
-        <v>102.8780332334752</v>
+        <v>102.878043272212</v>
       </c>
       <c r="N65" t="n">
-        <v>99.21869505775395</v>
+        <v>99.21869314315774</v>
       </c>
       <c r="O65" t="n">
-        <v>150.6938083422704</v>
+        <v>150.6938306768409</v>
       </c>
       <c r="P65" t="n">
-        <v>891.8023236596122</v>
+        <v>891.8021108387103</v>
       </c>
       <c r="Q65" t="n">
-        <v>121.1944673978549</v>
+        <v>121.1944771402074</v>
       </c>
       <c r="R65" t="n">
-        <v>669.5666374540945</v>
+        <v>669.5667202959797</v>
       </c>
     </row>
     <row r="66">
@@ -3996,22 +3996,22 @@
         <v>2.8</v>
       </c>
       <c r="M66" t="n">
-        <v>101.9464260691198</v>
+        <v>101.946442542177</v>
       </c>
       <c r="N66" t="n">
-        <v>104.9790270042161</v>
+        <v>104.9790231345184</v>
       </c>
       <c r="O66" t="n">
-        <v>152.5572373314974</v>
+        <v>152.5572637436995</v>
       </c>
       <c r="P66" t="n">
-        <v>945.5802888567541</v>
+        <v>945.5801149938666</v>
       </c>
       <c r="Q66" t="n">
-        <v>142.2389906840362</v>
+        <v>142.2389859980242</v>
       </c>
       <c r="R66" t="n">
-        <v>894.9831657704783</v>
+        <v>894.9833193511681</v>
       </c>
     </row>
     <row r="67">
@@ -4052,22 +4052,22 @@
         <v>2.86</v>
       </c>
       <c r="M67" t="n">
-        <v>104.3474257034366</v>
+        <v>104.3474393352829</v>
       </c>
       <c r="N67" t="n">
-        <v>103.3505952805919</v>
+        <v>103.3506162622817</v>
       </c>
       <c r="O67" t="n">
-        <v>156.196650454587</v>
+        <v>156.1966358823299</v>
       </c>
       <c r="P67" t="n">
-        <v>1025.49271106536</v>
+        <v>1025.492490308808</v>
       </c>
       <c r="Q67" t="n">
-        <v>131.135065826541</v>
+        <v>131.1350793206077</v>
       </c>
       <c r="R67" t="n">
-        <v>1086.872658396869</v>
+        <v>1086.872717777688</v>
       </c>
     </row>
     <row r="68">
@@ -4108,22 +4108,22 @@
         <v>2.55</v>
       </c>
       <c r="M68" s="3" t="n">
-        <v>106.5134692276869</v>
+        <v>106.5134826520623</v>
       </c>
       <c r="N68" s="3" t="n">
-        <v>109.4835590636833</v>
+        <v>109.4835607407023</v>
       </c>
       <c r="O68" s="3" t="n">
-        <v>154.0140857427668</v>
+        <v>154.0140759254842</v>
       </c>
       <c r="P68" s="3" t="n">
-        <v>1369.520182923256</v>
+        <v>1369.519709299506</v>
       </c>
       <c r="Q68" s="3" t="n">
-        <v>132.947182530961</v>
+        <v>132.9471953871984</v>
       </c>
       <c r="R68" s="3" t="n">
-        <v>1437.457312791659</v>
+        <v>1437.457180900158</v>
       </c>
     </row>
     <row r="69">
@@ -4164,22 +4164,22 @@
         <v>2.6</v>
       </c>
       <c r="M69" s="3" t="n">
-        <v>100.8568654673158</v>
+        <v>100.8568806399331</v>
       </c>
       <c r="N69" s="3" t="n">
-        <v>106.6442544409175</v>
+        <v>106.6442597701652</v>
       </c>
       <c r="O69" s="3" t="n">
-        <v>157.8706692190119</v>
+        <v>157.8706881906564</v>
       </c>
       <c r="P69" s="3" t="n">
-        <v>1432.372483137599</v>
+        <v>1432.372199262938</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>125.1881263308945</v>
+        <v>125.1881277090199</v>
       </c>
       <c r="R69" s="3" t="n">
-        <v>1518.658692006362</v>
+        <v>1518.658518602595</v>
       </c>
     </row>
     <row r="70">
@@ -4220,22 +4220,22 @@
         <v>2.67</v>
       </c>
       <c r="M70" t="n">
-        <v>96.65414005795267</v>
+        <v>96.65414213092112</v>
       </c>
       <c r="N70" t="n">
-        <v>106.8964805991708</v>
+        <v>106.8964850008862</v>
       </c>
       <c r="O70" t="n">
-        <v>155.2863456955157</v>
+        <v>155.2863539863279</v>
       </c>
       <c r="P70" t="n">
-        <v>1427.787947590759</v>
+        <v>1427.787770239212</v>
       </c>
       <c r="Q70" t="n">
-        <v>126.6162505303238</v>
+        <v>126.6162626683864</v>
       </c>
       <c r="R70" t="n">
-        <v>1485.445896824275</v>
+        <v>1485.44604964789</v>
       </c>
     </row>
     <row r="71">
@@ -4276,22 +4276,22 @@
         <v>2.62</v>
       </c>
       <c r="M71" t="n">
-        <v>93.06512352714147</v>
+        <v>93.06513827681655</v>
       </c>
       <c r="N71" t="n">
-        <v>101.8015107702597</v>
+        <v>101.8015159409412</v>
       </c>
       <c r="O71" t="n">
-        <v>146.2495275766464</v>
+        <v>146.2495595043298</v>
       </c>
       <c r="P71" t="n">
-        <v>1542.611724547781</v>
+        <v>1542.611643384497</v>
       </c>
       <c r="Q71" t="n">
-        <v>121.2082214281356</v>
+        <v>121.2082005388248</v>
       </c>
       <c r="R71" t="n">
-        <v>1570.877965792447</v>
+        <v>1570.878007110987</v>
       </c>
     </row>
     <row r="72">
@@ -4332,22 +4332,22 @@
         <v>2.75</v>
       </c>
       <c r="M72" t="n">
-        <v>109.0474061271542</v>
+        <v>109.0474118203171</v>
       </c>
       <c r="N72" t="n">
-        <v>106.6989993915202</v>
+        <v>106.6990027521929</v>
       </c>
       <c r="O72" t="n">
-        <v>150.1763164341159</v>
+        <v>150.1763271195221</v>
       </c>
       <c r="P72" t="n">
-        <v>1570.258243922381</v>
+        <v>1570.257858291615</v>
       </c>
       <c r="Q72" t="n">
-        <v>140.307324945927</v>
+        <v>140.3073561071203</v>
       </c>
       <c r="R72" t="n">
-        <v>1624.445825661683</v>
+        <v>1624.445866142519</v>
       </c>
     </row>
     <row r="73">
@@ -4388,22 +4388,22 @@
         <v>2.65</v>
       </c>
       <c r="M73" t="n">
-        <v>125.7098559914967</v>
+        <v>125.7098690524305</v>
       </c>
       <c r="N73" t="n">
-        <v>107.6992555504447</v>
+        <v>107.6992528118961</v>
       </c>
       <c r="O73" t="n">
-        <v>148.0565108969866</v>
+        <v>148.0565407562985</v>
       </c>
       <c r="P73" t="n">
-        <v>1623.653286321298</v>
+        <v>1623.652864063143</v>
       </c>
       <c r="Q73" t="n">
-        <v>147.2911067875705</v>
+        <v>147.2911058843931</v>
       </c>
       <c r="R73" t="n">
-        <v>1678.6779916422</v>
+        <v>1678.677850349775</v>
       </c>
     </row>
     <row r="74">
@@ -4444,22 +4444,22 @@
         <v>2.7</v>
       </c>
       <c r="M74" t="n">
-        <v>118.6266657810648</v>
+        <v>118.6266893729437</v>
       </c>
       <c r="N74" t="n">
-        <v>104.8459897799837</v>
+        <v>104.8459932826389</v>
       </c>
       <c r="O74" t="n">
-        <v>144.705423382137</v>
+        <v>144.7054199724683</v>
       </c>
       <c r="P74" t="n">
-        <v>1990.636488033048</v>
+        <v>1990.636156706497</v>
       </c>
       <c r="Q74" t="n">
-        <v>134.9004174289825</v>
+        <v>134.9004201719627</v>
       </c>
       <c r="R74" t="n">
-        <v>1732.326695848922</v>
+        <v>1732.326917211831</v>
       </c>
     </row>
     <row r="75">
@@ -4500,22 +4500,22 @@
         <v>3.08</v>
       </c>
       <c r="M75" t="n">
-        <v>124.3828682647533</v>
+        <v>124.3828714927729</v>
       </c>
       <c r="N75" t="n">
-        <v>106.6853113858976</v>
+        <v>106.6853099992759</v>
       </c>
       <c r="O75" t="n">
-        <v>147.6796498156545</v>
+        <v>147.679658898804</v>
       </c>
       <c r="P75" t="n">
-        <v>2138.413482829195</v>
+        <v>2138.413102080342</v>
       </c>
       <c r="Q75" t="n">
-        <v>142.3099284798053</v>
+        <v>142.3099126262222</v>
       </c>
       <c r="R75" t="n">
-        <v>1689.241415901625</v>
+        <v>1689.241579833105</v>
       </c>
     </row>
     <row r="76">
@@ -4556,22 +4556,22 @@
         <v>3.24</v>
       </c>
       <c r="M76" t="n">
-        <v>127.7719544961434</v>
+        <v>127.7719679280234</v>
       </c>
       <c r="N76" t="n">
-        <v>103.6075579207537</v>
+        <v>103.6075708831288</v>
       </c>
       <c r="O76" t="n">
-        <v>149.2602324496376</v>
+        <v>149.2602247945665</v>
       </c>
       <c r="P76" t="n">
-        <v>1975.662735012843</v>
+        <v>1975.662616023761</v>
       </c>
       <c r="Q76" t="n">
-        <v>146.6408425913201</v>
+        <v>146.6408211243747</v>
       </c>
       <c r="R76" t="n">
-        <v>1631.551092475338</v>
+        <v>1631.550983235458</v>
       </c>
     </row>
     <row r="77">
@@ -4612,22 +4612,22 @@
         <v>3.11</v>
       </c>
       <c r="M77" t="n">
-        <v>125.2157924435858</v>
+        <v>125.215816499571</v>
       </c>
       <c r="N77" t="n">
-        <v>101.1132741029564</v>
+        <v>101.1132736499552</v>
       </c>
       <c r="O77" t="n">
-        <v>149.6567013347409</v>
+        <v>149.6567281110611</v>
       </c>
       <c r="P77" t="n">
-        <v>2010.606301140026</v>
+        <v>2010.606075418621</v>
       </c>
       <c r="Q77" t="n">
-        <v>147.4509375215345</v>
+        <v>147.4509468623796</v>
       </c>
       <c r="R77" t="n">
-        <v>1873.307029744744</v>
+        <v>1873.307068361115</v>
       </c>
     </row>
     <row r="78">
@@ -4668,22 +4668,22 @@
         <v>3.23</v>
       </c>
       <c r="M78" t="n">
-        <v>129.0394691340401</v>
+        <v>129.0394799666029</v>
       </c>
       <c r="N78" t="n">
-        <v>101.7027976743278</v>
+        <v>101.7028048443715</v>
       </c>
       <c r="O78" t="n">
-        <v>142.8797286901632</v>
+        <v>142.8797371505479</v>
       </c>
       <c r="P78" t="n">
-        <v>1901.29252772114</v>
+        <v>1901.292045923983</v>
       </c>
       <c r="Q78" t="n">
-        <v>144.8917920758414</v>
+        <v>144.8917616515182</v>
       </c>
       <c r="R78" t="n">
-        <v>1796.757238457163</v>
+        <v>1796.757456736691</v>
       </c>
     </row>
     <row r="79">
@@ -4724,22 +4724,22 @@
         <v>3.28</v>
       </c>
       <c r="M79" t="n">
-        <v>130.9031057293707</v>
+        <v>130.9031266115862</v>
       </c>
       <c r="N79" t="n">
-        <v>92.00478361023052</v>
+        <v>92.00478472018239</v>
       </c>
       <c r="O79" t="n">
-        <v>145.2745232828059</v>
+        <v>145.274532058284</v>
       </c>
       <c r="P79" t="n">
-        <v>1853.515430259787</v>
+        <v>1853.515081966749</v>
       </c>
       <c r="Q79" t="n">
-        <v>142.9890759021614</v>
+        <v>142.9890612419484</v>
       </c>
       <c r="R79" t="n">
-        <v>1578.897128919345</v>
+        <v>1578.89709180792</v>
       </c>
     </row>
     <row r="80">
@@ -4780,22 +4780,22 @@
         <v>3.17</v>
       </c>
       <c r="M80" t="n">
-        <v>127.503385962521</v>
+        <v>127.503401923989</v>
       </c>
       <c r="N80" t="n">
-        <v>84.13026946447994</v>
+        <v>84.13028444737797</v>
       </c>
       <c r="O80" t="n">
-        <v>143.5884932477945</v>
+        <v>143.5884831459239</v>
       </c>
       <c r="P80" t="n">
-        <v>2143.398125756555</v>
+        <v>2143.397347302599</v>
       </c>
       <c r="Q80" t="n">
-        <v>141.6220312034214</v>
+        <v>141.6220334086307</v>
       </c>
       <c r="R80" t="n">
-        <v>1552.024380529356</v>
+        <v>1552.024397936409</v>
       </c>
     </row>
     <row r="81">
@@ -4836,22 +4836,22 @@
         <v>3.19</v>
       </c>
       <c r="M81" s="3" t="n">
-        <v>136.0921752528854</v>
+        <v>136.0922021367026</v>
       </c>
       <c r="N81" s="3" t="n">
-        <v>97.41067256009983</v>
+        <v>97.41068079810556</v>
       </c>
       <c r="O81" s="3" t="n">
-        <v>147.1370272079248</v>
+        <v>147.1370173578062</v>
       </c>
       <c r="P81" s="3" t="n">
-        <v>2199.753013519288</v>
+        <v>2199.752444469665</v>
       </c>
       <c r="Q81" s="3" t="n">
-        <v>152.0642249553502</v>
+        <v>152.0642267342895</v>
       </c>
       <c r="R81" s="3" t="n">
-        <v>1649.044066610918</v>
+        <v>1649.044093072782</v>
       </c>
     </row>
     <row r="82">
@@ -4892,22 +4892,22 @@
         <v>3.37</v>
       </c>
       <c r="M82" t="n">
-        <v>135.1539914419436</v>
+        <v>135.1540218749277</v>
       </c>
       <c r="N82" t="n">
-        <v>89.70233743387915</v>
+        <v>89.7023328318591</v>
       </c>
       <c r="O82" t="n">
-        <v>144.0130166859808</v>
+        <v>144.0130211202435</v>
       </c>
       <c r="P82" t="n">
-        <v>2360.046258841667</v>
+        <v>2360.045511893407</v>
       </c>
       <c r="Q82" t="n">
-        <v>154.7132281407453</v>
+        <v>154.7132241764373</v>
       </c>
       <c r="R82" t="n">
-        <v>1450.170032265938</v>
+        <v>1450.170089153185</v>
       </c>
     </row>
     <row r="83">
@@ -4948,22 +4948,22 @@
         <v>3.58</v>
       </c>
       <c r="M83" t="n">
-        <v>140.3524053379632</v>
+        <v>140.3524224500671</v>
       </c>
       <c r="N83" t="n">
-        <v>97.44535631534666</v>
+        <v>97.44535761225347</v>
       </c>
       <c r="O83" t="n">
-        <v>148.1641863680547</v>
+        <v>148.1642029091576</v>
       </c>
       <c r="P83" t="n">
-        <v>2430.506272596513</v>
+        <v>2430.505755508718</v>
       </c>
       <c r="Q83" t="n">
-        <v>157.7723797804005</v>
+        <v>157.7723755403084</v>
       </c>
       <c r="R83" t="n">
-        <v>1402.267960622868</v>
+        <v>1402.268075415556</v>
       </c>
     </row>
     <row r="84">
@@ -5004,22 +5004,22 @@
         <v>3.51</v>
       </c>
       <c r="M84" t="n">
-        <v>137.0036277819553</v>
+        <v>137.0036497779476</v>
       </c>
       <c r="N84" t="n">
-        <v>91.90437612571735</v>
+        <v>91.90438365653037</v>
       </c>
       <c r="O84" t="n">
-        <v>144.5731893052734</v>
+        <v>144.573194165164</v>
       </c>
       <c r="P84" t="n">
-        <v>2521.896737379279</v>
+        <v>2521.896134493657</v>
       </c>
       <c r="Q84" t="n">
-        <v>155.818194790208</v>
+        <v>155.8181814595404</v>
       </c>
       <c r="R84" t="n">
-        <v>1449.937387109367</v>
+        <v>1449.937390891817</v>
       </c>
     </row>
     <row r="85">
@@ -5060,22 +5060,22 @@
         <v>3.6</v>
       </c>
       <c r="M85" t="n">
-        <v>143.8155597518324</v>
+        <v>143.8155830679714</v>
       </c>
       <c r="N85" t="n">
-        <v>94.15386987235217</v>
+        <v>94.15386858448662</v>
       </c>
       <c r="O85" t="n">
-        <v>144.7392360699459</v>
+        <v>144.7392477696232</v>
       </c>
       <c r="P85" t="n">
-        <v>2524.528922208436</v>
+        <v>2524.528328069109</v>
       </c>
       <c r="Q85" t="n">
-        <v>165.7911047538583</v>
+        <v>165.7911215718216</v>
       </c>
       <c r="R85" t="n">
-        <v>1431.853444663133</v>
+        <v>1431.853657118044</v>
       </c>
     </row>
     <row r="86">
@@ -5116,22 +5116,22 @@
         <v>3.68</v>
       </c>
       <c r="M86" t="n">
-        <v>142.0356848761494</v>
+        <v>142.0356957327137</v>
       </c>
       <c r="N86" t="n">
-        <v>92.57399445457388</v>
+        <v>92.57400481492172</v>
       </c>
       <c r="O86" t="n">
-        <v>139.765782716316</v>
+        <v>139.7657974088378</v>
       </c>
       <c r="P86" t="n">
-        <v>2056.305667523419</v>
+        <v>2056.305166469143</v>
       </c>
       <c r="Q86" t="n">
-        <v>159.2857087054996</v>
+        <v>159.2857002228904</v>
       </c>
       <c r="R86" t="n">
-        <v>1343.501077217149</v>
+        <v>1343.501068241441</v>
       </c>
     </row>
     <row r="87">
@@ -5172,22 +5172,22 @@
         <v>3.67</v>
       </c>
       <c r="M87" t="n">
-        <v>152.1997249681246</v>
+        <v>152.1997342371232</v>
       </c>
       <c r="N87" t="n">
-        <v>118.7453939250492</v>
+        <v>118.7453996526787</v>
       </c>
       <c r="O87" t="n">
-        <v>139.6934056374245</v>
+        <v>139.6934256962023</v>
       </c>
       <c r="P87" t="n">
-        <v>1917.443309347392</v>
+        <v>1917.442815152799</v>
       </c>
       <c r="Q87" t="n">
-        <v>170.3776678536209</v>
+        <v>170.3776565135157</v>
       </c>
       <c r="R87" t="n">
-        <v>1391.265739748291</v>
+        <v>1391.265865353072</v>
       </c>
     </row>
     <row r="88">
@@ -5228,22 +5228,22 @@
         <v>3.85</v>
       </c>
       <c r="M88" t="n">
-        <v>156.2847697768419</v>
+        <v>156.2847952317414</v>
       </c>
       <c r="N88" t="n">
-        <v>114.4358123072375</v>
+        <v>114.4358196593071</v>
       </c>
       <c r="O88" t="n">
-        <v>144.1660577276409</v>
+        <v>144.1660696774446</v>
       </c>
       <c r="P88" t="n">
-        <v>2005.958425431494</v>
+        <v>2005.958015043514</v>
       </c>
       <c r="Q88" t="n">
-        <v>168.673436061376</v>
+        <v>168.6734177138054</v>
       </c>
       <c r="R88" t="n">
-        <v>1292.435893061061</v>
+        <v>1292.435945218485</v>
       </c>
     </row>
     <row r="89">
@@ -5284,22 +5284,22 @@
         <v>4.38</v>
       </c>
       <c r="M89" t="n">
-        <v>156.0117143799631</v>
+        <v>156.011732482753</v>
       </c>
       <c r="N89" t="n">
-        <v>129.1144019895052</v>
+        <v>129.1144042859107</v>
       </c>
       <c r="O89" t="n">
-        <v>149.7028464500386</v>
+        <v>149.7028447794129</v>
       </c>
       <c r="P89" t="n">
-        <v>1856.20774990973</v>
+        <v>1856.207543266642</v>
       </c>
       <c r="Q89" t="n">
-        <v>177.1733126513817</v>
+        <v>177.1733101417254</v>
       </c>
       <c r="R89" t="n">
-        <v>1191.190034183048</v>
+        <v>1191.190025399982</v>
       </c>
     </row>
     <row r="90">
@@ -5340,22 +5340,22 @@
         <v>4.17</v>
       </c>
       <c r="M90" t="n">
-        <v>156.1560156718381</v>
+        <v>156.1560408092938</v>
       </c>
       <c r="N90" t="n">
-        <v>118.2835112999915</v>
+        <v>118.283524834238</v>
       </c>
       <c r="O90" t="n">
-        <v>155.8575694800351</v>
+        <v>155.8575872430038</v>
       </c>
       <c r="P90" t="n">
-        <v>1851.6147214253</v>
+        <v>1851.614237418138</v>
       </c>
       <c r="Q90" t="n">
-        <v>180.8854378689784</v>
+        <v>180.8854342515725</v>
       </c>
       <c r="R90" t="n">
-        <v>1048.465605096166</v>
+        <v>1048.465578952477</v>
       </c>
     </row>
     <row r="91">
@@ -5396,22 +5396,22 @@
         <v>4.26</v>
       </c>
       <c r="M91" t="n">
-        <v>147.4005932945471</v>
+        <v>147.4006060525951</v>
       </c>
       <c r="N91" t="n">
-        <v>103.1306788245896</v>
+        <v>103.1306859706293</v>
       </c>
       <c r="O91" t="n">
-        <v>152.6327915660292</v>
+        <v>152.6327991729655</v>
       </c>
       <c r="P91" t="n">
-        <v>1675.867821612057</v>
+        <v>1675.867637920882</v>
       </c>
       <c r="Q91" t="n">
-        <v>167.5301754596397</v>
+        <v>167.5301686853534</v>
       </c>
       <c r="R91" t="n">
-        <v>845.9729662705197</v>
+        <v>845.9731077316487</v>
       </c>
     </row>
     <row r="92">
@@ -5452,22 +5452,22 @@
         <v>3.88</v>
       </c>
       <c r="M92" t="n">
-        <v>154.4707174089193</v>
+        <v>154.4707228884041</v>
       </c>
       <c r="N92" t="n">
-        <v>105.5314663453258</v>
+        <v>105.5314774565112</v>
       </c>
       <c r="O92" t="n">
-        <v>155.7340724047196</v>
+        <v>155.7340619024395</v>
       </c>
       <c r="P92" t="n">
-        <v>1903.561180203848</v>
+        <v>1903.560761534813</v>
       </c>
       <c r="Q92" t="n">
-        <v>172.7816771712098</v>
+        <v>172.7816665478998</v>
       </c>
       <c r="R92" t="n">
-        <v>827.1238366893643</v>
+        <v>827.1238104383965</v>
       </c>
     </row>
     <row r="93">
@@ -5508,22 +5508,22 @@
         <v>3.98</v>
       </c>
       <c r="M93" s="3" t="n">
-        <v>157.4945446568432</v>
+        <v>157.4945610472005</v>
       </c>
       <c r="N93" s="3" t="n">
-        <v>110.1823830248428</v>
+        <v>110.1823857934647</v>
       </c>
       <c r="O93" s="3" t="n">
-        <v>155.7363328379108</v>
+        <v>155.736327997894</v>
       </c>
       <c r="P93" s="3" t="n">
-        <v>1814.667728853732</v>
+        <v>1814.667326486149</v>
       </c>
       <c r="Q93" s="3" t="n">
-        <v>175.9636985930933</v>
+        <v>175.9636868110021</v>
       </c>
       <c r="R93" s="3" t="n">
-        <v>751.774680366659</v>
+        <v>751.774689222214</v>
       </c>
     </row>
     <row r="94">
@@ -5564,22 +5564,22 @@
         <v>4.41</v>
       </c>
       <c r="M94" t="n">
-        <v>151.2032175790608</v>
+        <v>151.2032229527444</v>
       </c>
       <c r="N94" t="n">
-        <v>100.0466232436894</v>
+        <v>100.04663427914</v>
       </c>
       <c r="O94" t="n">
-        <v>150.897708277856</v>
+        <v>150.8977044026503</v>
       </c>
       <c r="P94" t="n">
-        <v>1773.936156256385</v>
+        <v>1773.935840614711</v>
       </c>
       <c r="Q94" t="n">
-        <v>164.0738779530403</v>
+        <v>164.0738778288424</v>
       </c>
       <c r="R94" t="n">
-        <v>611.3913195408352</v>
+        <v>611.3913522543892</v>
       </c>
     </row>
     <row r="95">
@@ -5620,22 +5620,22 @@
         <v>4.37</v>
       </c>
       <c r="M95" t="n">
-        <v>157.944645927172</v>
+        <v>157.9446777514006</v>
       </c>
       <c r="N95" t="n">
-        <v>107.0110486677763</v>
+        <v>107.0110527842983</v>
       </c>
       <c r="O95" t="n">
-        <v>150.286480629819</v>
+        <v>150.2864897898888</v>
       </c>
       <c r="P95" t="n">
-        <v>1691.667386758266</v>
+        <v>1691.66683728684</v>
       </c>
       <c r="Q95" t="n">
-        <v>172.9320475410137</v>
+        <v>172.9320537450108</v>
       </c>
       <c r="R95" t="n">
-        <v>717.9480806720017</v>
+        <v>717.9480429495858</v>
       </c>
     </row>
     <row r="96">
@@ -5676,22 +5676,22 @@
         <v>4.11</v>
       </c>
       <c r="M96" t="n">
-        <v>161.2597276613734</v>
+        <v>161.2597436599056</v>
       </c>
       <c r="N96" t="n">
-        <v>103.1780550043311</v>
+        <v>103.1780544634575</v>
       </c>
       <c r="O96" t="n">
-        <v>156.5294561923434</v>
+        <v>156.5294605238562</v>
       </c>
       <c r="P96" t="n">
-        <v>1896.300090005079</v>
+        <v>1896.299650823623</v>
       </c>
       <c r="Q96" t="n">
-        <v>177.027938010687</v>
+        <v>177.0279495761934</v>
       </c>
       <c r="R96" t="n">
-        <v>798.4068724304198</v>
+        <v>798.4069345829904</v>
       </c>
     </row>
     <row r="97">
@@ -5732,22 +5732,22 @@
         <v>4.07</v>
       </c>
       <c r="M97" t="n">
-        <v>160.0503117281062</v>
+        <v>160.0503362510775</v>
       </c>
       <c r="N97" t="n">
-        <v>110.9615835477329</v>
+        <v>110.9615827618592</v>
       </c>
       <c r="O97" t="n">
-        <v>157.2009547602877</v>
+        <v>157.200969143304</v>
       </c>
       <c r="P97" t="n">
-        <v>1917.380695108568</v>
+        <v>1917.380041535468</v>
       </c>
       <c r="Q97" t="n">
-        <v>177.307674440675</v>
+        <v>177.3076463688183</v>
       </c>
       <c r="R97" t="n">
-        <v>822.0042343554267</v>
+        <v>822.0043221843986</v>
       </c>
     </row>
     <row r="98">
@@ -5788,22 +5788,22 @@
         <v>3.8</v>
       </c>
       <c r="M98" t="n">
-        <v>158.8606029377696</v>
+        <v>158.8606228310599</v>
       </c>
       <c r="N98" t="n">
-        <v>104.832871071772</v>
+        <v>104.8328678462992</v>
       </c>
       <c r="O98" t="n">
-        <v>167.4155147027576</v>
+        <v>167.4155226548303</v>
       </c>
       <c r="P98" t="n">
-        <v>1975.640457835304</v>
+        <v>1975.639876536299</v>
       </c>
       <c r="Q98" t="n">
-        <v>171.6035009193153</v>
+        <v>171.6034975535558</v>
       </c>
       <c r="R98" t="n">
-        <v>813.2539705461365</v>
+        <v>813.2539704739573</v>
       </c>
     </row>
     <row r="99">
@@ -5844,22 +5844,22 @@
         <v>3.91</v>
       </c>
       <c r="M99" t="n">
-        <v>156.5803053440524</v>
+        <v>156.5803234839629</v>
       </c>
       <c r="N99" t="n">
-        <v>104.416189430124</v>
+        <v>104.4162001632384</v>
       </c>
       <c r="O99" t="n">
-        <v>167.776709069591</v>
+        <v>167.7766952525492</v>
       </c>
       <c r="P99" t="n">
-        <v>1921.947154911697</v>
+        <v>1921.946699143884</v>
       </c>
       <c r="Q99" t="n">
-        <v>160.8391240427291</v>
+        <v>160.8391308698273</v>
       </c>
       <c r="R99" t="n">
-        <v>775.8855804551943</v>
+        <v>775.885589939582</v>
       </c>
     </row>
     <row r="100">
@@ -5900,22 +5900,22 @@
         <v>3.91</v>
       </c>
       <c r="M100" t="n">
-        <v>154.4604585321645</v>
+        <v>154.4604738939129</v>
       </c>
       <c r="N100" t="n">
-        <v>105.1575105913113</v>
+        <v>105.1575149686814</v>
       </c>
       <c r="O100" t="n">
-        <v>170.1199831061443</v>
+        <v>170.1199849398316</v>
       </c>
       <c r="P100" t="n">
-        <v>1928.227933033479</v>
+        <v>1928.227573529125</v>
       </c>
       <c r="Q100" t="n">
-        <v>163.5448020998727</v>
+        <v>163.5447998509028</v>
       </c>
       <c r="R100" t="n">
-        <v>850.2833448301136</v>
+        <v>850.2833940958789</v>
       </c>
     </row>
     <row r="101">
@@ -5956,22 +5956,22 @@
         <v>3.73</v>
       </c>
       <c r="M101" t="n">
-        <v>151.1413688103023</v>
+        <v>151.1413974320196</v>
       </c>
       <c r="N101" t="n">
-        <v>107.0643080172437</v>
+        <v>107.0643140144907</v>
       </c>
       <c r="O101" t="n">
-        <v>172.3313565043006</v>
+        <v>172.3313586052563</v>
       </c>
       <c r="P101" t="n">
-        <v>1871.124012716082</v>
+        <v>1871.123748800087</v>
       </c>
       <c r="Q101" t="n">
-        <v>168.387588707094</v>
+        <v>168.3876110305044</v>
       </c>
       <c r="R101" t="n">
-        <v>895.4035451051656</v>
+        <v>895.4035676432463</v>
       </c>
     </row>
     <row r="102">
@@ -6012,22 +6012,22 @@
         <v>3.7</v>
       </c>
       <c r="M102" t="n">
-        <v>147.6786385003953</v>
+        <v>147.6786577899014</v>
       </c>
       <c r="N102" t="n">
-        <v>104.4072317264568</v>
+        <v>104.4072419754525</v>
       </c>
       <c r="O102" t="n">
-        <v>167.3140789629893</v>
+        <v>167.314083173723</v>
       </c>
       <c r="P102" t="n">
-        <v>1931.984124667843</v>
+        <v>1931.983536056777</v>
       </c>
       <c r="Q102" t="n">
-        <v>160.0635290256845</v>
+        <v>160.0635265683348</v>
       </c>
       <c r="R102" t="n">
-        <v>919.1695578825424</v>
+        <v>919.1696017850372</v>
       </c>
     </row>
     <row r="103">
@@ -6068,22 +6068,22 @@
         <v>3.85</v>
       </c>
       <c r="M103" t="n">
-        <v>150.5253891380518</v>
+        <v>150.5254069841397</v>
       </c>
       <c r="N103" t="n">
-        <v>106.0914140016929</v>
+        <v>106.091429096657</v>
       </c>
       <c r="O103" t="n">
-        <v>169.4970592034264</v>
+        <v>169.4970732723172</v>
       </c>
       <c r="P103" t="n">
-        <v>2024.134883944762</v>
+        <v>2024.13434496858</v>
       </c>
       <c r="Q103" t="n">
-        <v>159.015485437679</v>
+        <v>159.0154743856061</v>
       </c>
       <c r="R103" t="n">
-        <v>787.4314767818655</v>
+        <v>787.431467990896</v>
       </c>
     </row>
     <row r="104">
@@ -6124,22 +6124,22 @@
         <v>3.84</v>
       </c>
       <c r="M104" t="n">
-        <v>161.8181180458683</v>
+        <v>161.8181464816108</v>
       </c>
       <c r="N104" t="n">
-        <v>116.2393646140737</v>
+        <v>116.2393726874334</v>
       </c>
       <c r="O104" t="n">
-        <v>165.8750196369966</v>
+        <v>165.8750286702923</v>
       </c>
       <c r="P104" t="n">
-        <v>2104.136078617876</v>
+        <v>2104.13536121824</v>
       </c>
       <c r="Q104" t="n">
-        <v>170.3048973171494</v>
+        <v>170.3048815186974</v>
       </c>
       <c r="R104" t="n">
-        <v>870.6468824581668</v>
+        <v>870.6469528373907</v>
       </c>
     </row>
     <row r="105">
@@ -6180,22 +6180,22 @@
         <v>3.84</v>
       </c>
       <c r="M105" s="3" t="n">
-        <v>163.9460266345995</v>
+        <v>163.946040793096</v>
       </c>
       <c r="N105" s="3" t="n">
-        <v>110.6407559477275</v>
+        <v>110.6407626594762</v>
       </c>
       <c r="O105" s="3" t="n">
-        <v>166.6150386349272</v>
+        <v>166.6150546334441</v>
       </c>
       <c r="P105" s="3" t="n">
-        <v>2166.051119134786</v>
+        <v>2166.050690345036</v>
       </c>
       <c r="Q105" s="3" t="n">
-        <v>169.982571640477</v>
+        <v>169.9825443088085</v>
       </c>
       <c r="R105" s="3" t="n">
-        <v>779.5727539685746</v>
+        <v>779.5728742682577</v>
       </c>
     </row>
     <row r="106">
@@ -6236,22 +6236,22 @@
         <v>3.97</v>
       </c>
       <c r="M106" t="n">
-        <v>162.4351118001</v>
+        <v>162.4351201976528</v>
       </c>
       <c r="N106" t="n">
-        <v>109.9229558423184</v>
+        <v>109.9229690915213</v>
       </c>
       <c r="O106" t="n">
-        <v>168.0613154536782</v>
+        <v>168.0613248005854</v>
       </c>
       <c r="P106" t="n">
-        <v>2028.277611401438</v>
+        <v>2028.276984628586</v>
       </c>
       <c r="Q106" t="n">
-        <v>171.8372102500275</v>
+        <v>171.8372085517006</v>
       </c>
       <c r="R106" t="n">
-        <v>776.0769780209766</v>
+        <v>776.0770791113099</v>
       </c>
     </row>
     <row r="107">
@@ -6292,22 +6292,22 @@
         <v>4.11</v>
       </c>
       <c r="M107" t="n">
-        <v>167.9808528552626</v>
+        <v>167.9808672482432</v>
       </c>
       <c r="N107" t="n">
-        <v>111.003417858458</v>
+        <v>111.0034306839987</v>
       </c>
       <c r="O107" t="n">
-        <v>171.3636191457917</v>
+        <v>171.363611389377</v>
       </c>
       <c r="P107" t="n">
-        <v>1972.415589191406</v>
+        <v>1972.415021813679</v>
       </c>
       <c r="Q107" t="n">
-        <v>175.5912920595035</v>
+        <v>175.591293599187</v>
       </c>
       <c r="R107" t="n">
-        <v>767.9707774396338</v>
+        <v>767.9707522662866</v>
       </c>
     </row>
     <row r="108">
@@ -6348,22 +6348,22 @@
         <v>3.81</v>
       </c>
       <c r="M108" t="n">
-        <v>168.6215924336854</v>
+        <v>168.6216178106954</v>
       </c>
       <c r="N108" t="n">
-        <v>113.4489483571579</v>
+        <v>113.4489550224714</v>
       </c>
       <c r="O108" t="n">
-        <v>174.7788249727197</v>
+        <v>174.7788307730744</v>
       </c>
       <c r="P108" t="n">
-        <v>2001.508371927525</v>
+        <v>2001.50795664802</v>
       </c>
       <c r="Q108" t="n">
-        <v>172.1349216255006</v>
+        <v>172.1349252685141</v>
       </c>
       <c r="R108" t="n">
-        <v>803.698328822361</v>
+        <v>803.6984005322197</v>
       </c>
     </row>
     <row r="109">
@@ -6404,22 +6404,22 @@
         <v>3.74</v>
       </c>
       <c r="M109" t="n">
-        <v>170.3033330623022</v>
+        <v>170.3033487921466</v>
       </c>
       <c r="N109" t="n">
-        <v>112.585223746124</v>
+        <v>112.5852419240586</v>
       </c>
       <c r="O109" t="n">
-        <v>176.6482347824997</v>
+        <v>176.6482315052248</v>
       </c>
       <c r="P109" t="n">
-        <v>2069.770784798596</v>
+        <v>2069.770348235382</v>
       </c>
       <c r="Q109" t="n">
-        <v>173.4922474255485</v>
+        <v>173.4922434085601</v>
       </c>
       <c r="R109" t="n">
-        <v>851.8267788061371</v>
+        <v>851.8268068182614</v>
       </c>
     </row>
     <row r="110">
@@ -6460,22 +6460,22 @@
         <v>3.79</v>
       </c>
       <c r="M110" t="n">
-        <v>177.677753843991</v>
+        <v>177.6777799361356</v>
       </c>
       <c r="N110" t="n">
-        <v>114.2459989282934</v>
+        <v>114.2460082292982</v>
       </c>
       <c r="O110" t="n">
-        <v>181.9816168979239</v>
+        <v>181.9816203752637</v>
       </c>
       <c r="P110" t="n">
-        <v>2122.080634048682</v>
+        <v>2122.080083676341</v>
       </c>
       <c r="Q110" t="n">
-        <v>170.1439426792902</v>
+        <v>170.1438952311506</v>
       </c>
       <c r="R110" t="n">
-        <v>860.6895766229879</v>
+        <v>860.6896536831773</v>
       </c>
     </row>
     <row r="111">
@@ -6516,22 +6516,22 @@
         <v>3.86</v>
       </c>
       <c r="M111" t="n">
-        <v>181.7235688439439</v>
+        <v>181.7235867098164</v>
       </c>
       <c r="N111" t="n">
-        <v>113.734545437603</v>
+        <v>113.7345591890883</v>
       </c>
       <c r="O111" t="n">
-        <v>185.536633427889</v>
+        <v>185.5366406946688</v>
       </c>
       <c r="P111" t="n">
-        <v>2221.378534199563</v>
+        <v>2221.378010506524</v>
       </c>
       <c r="Q111" t="n">
-        <v>176.7683887403995</v>
+        <v>176.7683973461447</v>
       </c>
       <c r="R111" t="n">
-        <v>796.3759933570624</v>
+        <v>796.3760796770445</v>
       </c>
     </row>
     <row r="112">
@@ -6572,22 +6572,22 @@
         <v>3.85</v>
       </c>
       <c r="M112" t="n">
-        <v>187.7363919378955</v>
+        <v>187.7364151476058</v>
       </c>
       <c r="N112" t="n">
-        <v>114.0895607196094</v>
+        <v>114.0895687556391</v>
       </c>
       <c r="O112" t="n">
-        <v>183.7042899122306</v>
+        <v>183.7043010663418</v>
       </c>
       <c r="P112" t="n">
-        <v>2293.227348939291</v>
+        <v>2293.226902307346</v>
       </c>
       <c r="Q112" t="n">
-        <v>171.8898663783141</v>
+        <v>171.8898781130636</v>
       </c>
       <c r="R112" t="n">
-        <v>794.1983586397096</v>
+        <v>794.1983523660996</v>
       </c>
     </row>
     <row r="113">
@@ -6628,22 +6628,22 @@
         <v>3.97</v>
       </c>
       <c r="M113" t="n">
-        <v>186.2415217383354</v>
+        <v>186.2415574542452</v>
       </c>
       <c r="N113" t="n">
-        <v>117.578978319408</v>
+        <v>117.5789891397904</v>
       </c>
       <c r="O113" t="n">
-        <v>191.4531391431029</v>
+        <v>191.4531409590715</v>
       </c>
       <c r="P113" t="n">
-        <v>2264.582509241456</v>
+        <v>2264.582034443072</v>
       </c>
       <c r="Q113" t="n">
-        <v>174.1228216079261</v>
+        <v>174.1228367680561</v>
       </c>
       <c r="R113" t="n">
-        <v>897.3614477648473</v>
+        <v>897.3614652585613</v>
       </c>
     </row>
     <row r="114">
@@ -6684,22 +6684,22 @@
         <v>3.89</v>
       </c>
       <c r="M114" t="n">
-        <v>189.3714065752639</v>
+        <v>189.3714277126482</v>
       </c>
       <c r="N114" t="n">
-        <v>109.9133142809535</v>
+        <v>109.9133270897452</v>
       </c>
       <c r="O114" t="n">
-        <v>189.2828933933023</v>
+        <v>189.2828866489579</v>
       </c>
       <c r="P114" t="n">
-        <v>1983.216797758819</v>
+        <v>1983.216300796325</v>
       </c>
       <c r="Q114" t="n">
-        <v>169.1980530095952</v>
+        <v>169.1980380378934</v>
       </c>
       <c r="R114" t="n">
-        <v>1011.977808091033</v>
+        <v>1011.977918808155</v>
       </c>
     </row>
     <row r="115">
@@ -6740,22 +6740,22 @@
         <v>3.86</v>
       </c>
       <c r="M115" t="n">
-        <v>187.98423364973</v>
+        <v>187.9842536295329</v>
       </c>
       <c r="N115" t="n">
-        <v>108.1873445976669</v>
+        <v>108.1873499624312</v>
       </c>
       <c r="O115" t="n">
-        <v>189.8747522059505</v>
+        <v>189.8747632207307</v>
       </c>
       <c r="P115" t="n">
-        <v>2181.568735352678</v>
+        <v>2181.568270752414</v>
       </c>
       <c r="Q115" t="n">
-        <v>158.7202166271665</v>
+        <v>158.7202221423097</v>
       </c>
       <c r="R115" t="n">
-        <v>1054.21442793061</v>
+        <v>1054.214538265607</v>
       </c>
     </row>
     <row r="116">
@@ -6796,22 +6796,22 @@
         <v>3.72</v>
       </c>
       <c r="M116" t="n">
-        <v>198.3642323225625</v>
+        <v>198.3642589771528</v>
       </c>
       <c r="N116" t="n">
-        <v>112.6916323108251</v>
+        <v>112.6916430576564</v>
       </c>
       <c r="O116" t="n">
-        <v>198.1705198148931</v>
+        <v>198.17052139018</v>
       </c>
       <c r="P116" t="n">
-        <v>2150.626009102244</v>
+        <v>2150.62558983429</v>
       </c>
       <c r="Q116" t="n">
-        <v>156.3990038247527</v>
+        <v>156.3990048682616</v>
       </c>
       <c r="R116" t="n">
-        <v>987.5535624449169</v>
+        <v>987.5535627282324</v>
       </c>
     </row>
     <row r="117">
@@ -6852,22 +6852,22 @@
         <v>3.76</v>
       </c>
       <c r="M117" t="n">
-        <v>218.4672114301698</v>
+        <v>218.4672465256253</v>
       </c>
       <c r="N117" t="n">
-        <v>116.8869314728614</v>
+        <v>116.8869393153409</v>
       </c>
       <c r="O117" t="n">
-        <v>204.1825968153649</v>
+        <v>204.1826013327275</v>
       </c>
       <c r="P117" t="n">
-        <v>1857.219180597261</v>
+        <v>1857.218804482708</v>
       </c>
       <c r="Q117" t="n">
-        <v>167.4863781923875</v>
+        <v>167.4863805357737</v>
       </c>
       <c r="R117" t="n">
-        <v>899.8576017828602</v>
+        <v>899.8576601530294</v>
       </c>
     </row>
     <row r="118">
@@ -6908,22 +6908,22 @@
         <v>3.71</v>
       </c>
       <c r="M118" t="n">
-        <v>217.084985685251</v>
+        <v>217.0850242625682</v>
       </c>
       <c r="N118" t="n">
-        <v>114.387568863797</v>
+        <v>114.3875758886384</v>
       </c>
       <c r="O118" t="n">
-        <v>215.1839174545289</v>
+        <v>215.1839358232794</v>
       </c>
       <c r="P118" t="n">
-        <v>1755.431602677422</v>
+        <v>1755.431147456476</v>
       </c>
       <c r="Q118" t="n">
-        <v>157.284704027436</v>
+        <v>157.2847160222079</v>
       </c>
       <c r="R118" t="n">
-        <v>956.5224439207336</v>
+        <v>956.5224754500889</v>
       </c>
     </row>
     <row r="119">
@@ -6964,22 +6964,22 @@
         <v>3.92</v>
       </c>
       <c r="M119" s="3" t="n">
-        <v>214.6197324629407</v>
+        <v>214.6197748502982</v>
       </c>
       <c r="N119" s="3" t="n">
-        <v>114.9497432653407</v>
+        <v>114.9497559554171</v>
       </c>
       <c r="O119" s="3" t="n">
-        <v>217.8414956246776</v>
+        <v>217.841506345494</v>
       </c>
       <c r="P119" s="3" t="n">
-        <v>1787.642625541818</v>
+        <v>1787.642222246782</v>
       </c>
       <c r="Q119" s="3" t="n">
-        <v>153.5998677557627</v>
+        <v>153.5998665848855</v>
       </c>
       <c r="R119" s="3" t="n">
-        <v>959.4031005551029</v>
+        <v>959.4030720737331</v>
       </c>
     </row>
     <row r="120">
@@ -7020,22 +7020,22 @@
         <v>3.81</v>
       </c>
       <c r="M120" t="n">
-        <v>215.6979574481733</v>
+        <v>215.697991663738</v>
       </c>
       <c r="N120" t="n">
-        <v>116.1721184418543</v>
+        <v>116.172138875064</v>
       </c>
       <c r="O120" t="n">
-        <v>220.6866543595742</v>
+        <v>220.6866652041733</v>
       </c>
       <c r="P120" t="n">
-        <v>1797.779786151261</v>
+        <v>1797.779345263511</v>
       </c>
       <c r="Q120" t="n">
-        <v>152.3899955696756</v>
+        <v>152.3899900993696</v>
       </c>
       <c r="R120" t="n">
-        <v>993.3294278075415</v>
+        <v>993.3293736441871</v>
       </c>
     </row>
     <row r="121">
@@ -7076,22 +7076,22 @@
         <v>3.82</v>
       </c>
       <c r="M121" t="n">
-        <v>217.0264702619863</v>
+        <v>217.0264902470303</v>
       </c>
       <c r="N121" t="n">
-        <v>119.9192798580539</v>
+        <v>119.9192888473721</v>
       </c>
       <c r="O121" t="n">
-        <v>225.430234606078</v>
+        <v>225.4302423070495</v>
       </c>
       <c r="P121" t="n">
-        <v>2070.551041061854</v>
+        <v>2070.550469765984</v>
       </c>
       <c r="Q121" t="n">
-        <v>157.9848448702949</v>
+        <v>157.9848435740799</v>
       </c>
       <c r="R121" t="n">
-        <v>1097.910039940701</v>
+        <v>1097.909991751137</v>
       </c>
     </row>
     <row r="122">
@@ -7132,22 +7132,22 @@
         <v>3.81</v>
       </c>
       <c r="M122" t="n">
-        <v>212.2118138083424</v>
+        <v>212.2118363760427</v>
       </c>
       <c r="N122" t="n">
-        <v>114.8093942394136</v>
+        <v>114.8093967265777</v>
       </c>
       <c r="O122" t="n">
-        <v>228.1030596458334</v>
+        <v>228.1030641542739</v>
       </c>
       <c r="P122" t="n">
-        <v>1820.976781622559</v>
+        <v>1820.976330546101</v>
       </c>
       <c r="Q122" t="n">
-        <v>152.1773320696612</v>
+        <v>152.1773349260078</v>
       </c>
       <c r="R122" t="n">
-        <v>1040.086555188728</v>
+        <v>1040.086545295319</v>
       </c>
     </row>
     <row r="123">
@@ -7188,22 +7188,22 @@
         <v>3.79</v>
       </c>
       <c r="M123" t="n">
-        <v>216.5929820536581</v>
+        <v>216.5930139031723</v>
       </c>
       <c r="N123" t="n">
-        <v>119.7964563306469</v>
+        <v>119.7964669231029</v>
       </c>
       <c r="O123" t="n">
-        <v>237.6618745084309</v>
+        <v>237.6618802742814</v>
       </c>
       <c r="P123" t="n">
-        <v>1585.432731975401</v>
+        <v>1585.43224305334</v>
       </c>
       <c r="Q123" t="n">
-        <v>141.7103104240868</v>
+        <v>141.7103060475899</v>
       </c>
       <c r="R123" t="n">
-        <v>922.0197345426138</v>
+        <v>922.0198520583557</v>
       </c>
     </row>
     <row r="124">
@@ -7244,22 +7244,22 @@
         <v>3.77</v>
       </c>
       <c r="M124" s="3" t="n">
-        <v>209.1177919955135</v>
+        <v>209.1178154303584</v>
       </c>
       <c r="N124" s="3" t="n">
-        <v>116.7757685470425</v>
+        <v>116.775770022915</v>
       </c>
       <c r="O124" s="3" t="n">
-        <v>236.0877465189258</v>
+        <v>236.0877707945054</v>
       </c>
       <c r="P124" s="3" t="n">
-        <v>1570.898895362191</v>
+        <v>1570.898534810543</v>
       </c>
       <c r="Q124" s="3" t="n">
-        <v>139.0093969452183</v>
+        <v>139.009399262937</v>
       </c>
       <c r="R124" s="3" t="n">
-        <v>874.2068538965358</v>
+        <v>874.2068321744249</v>
       </c>
     </row>
     <row r="125">
@@ -7300,22 +7300,22 @@
         <v>3.66</v>
       </c>
       <c r="M125" t="n">
-        <v>210.3466992498875</v>
+        <v>210.34673162317</v>
       </c>
       <c r="N125" t="n">
-        <v>113.6282924930139</v>
+        <v>113.6283010860401</v>
       </c>
       <c r="O125" t="n">
-        <v>244.269011338987</v>
+        <v>244.2690289048057</v>
       </c>
       <c r="P125" t="n">
-        <v>1535.604031085544</v>
+        <v>1535.60361670344</v>
       </c>
       <c r="Q125" t="n">
-        <v>145.5124108617425</v>
+        <v>145.5124079201429</v>
       </c>
       <c r="R125" t="n">
-        <v>902.1749356119599</v>
+        <v>902.1749250794622</v>
       </c>
     </row>
     <row r="126">
@@ -7356,22 +7356,22 @@
         <v>3.52</v>
       </c>
       <c r="M126" t="n">
-        <v>204.5888547557031</v>
+        <v>204.5888778387027</v>
       </c>
       <c r="N126" t="n">
-        <v>111.5759485811558</v>
+        <v>111.5759575166995</v>
       </c>
       <c r="O126" t="n">
-        <v>252.516825580797</v>
+        <v>252.5168467746756</v>
       </c>
       <c r="P126" t="n">
-        <v>1588.890252364737</v>
+        <v>1588.889850188247</v>
       </c>
       <c r="Q126" t="n">
-        <v>143.6950189316279</v>
+        <v>143.6950077000719</v>
       </c>
       <c r="R126" t="n">
-        <v>878.885075902328</v>
+        <v>878.8850438356267</v>
       </c>
     </row>
     <row r="127">
@@ -7412,22 +7412,22 @@
         <v>3.47</v>
       </c>
       <c r="M127" t="n">
-        <v>202.7286774691023</v>
+        <v>202.7287057104048</v>
       </c>
       <c r="N127" t="n">
-        <v>116.7662997068193</v>
+        <v>116.7663095014319</v>
       </c>
       <c r="O127" t="n">
-        <v>263.7673908463964</v>
+        <v>263.7673909419136</v>
       </c>
       <c r="P127" t="n">
-        <v>1703.000403664495</v>
+        <v>1703.000009815427</v>
       </c>
       <c r="Q127" t="n">
-        <v>149.4021668901691</v>
+        <v>149.4021614647465</v>
       </c>
       <c r="R127" t="n">
-        <v>836.9484741903115</v>
+        <v>836.9484531978694</v>
       </c>
     </row>
     <row r="128">
@@ -7468,22 +7468,22 @@
         <v>3.37</v>
       </c>
       <c r="M128" t="n">
-        <v>196.7065493168377</v>
+        <v>196.7065746011206</v>
       </c>
       <c r="N128" t="n">
-        <v>116.4514049923657</v>
+        <v>116.451415268356</v>
       </c>
       <c r="O128" t="n">
-        <v>275.7312781685512</v>
+        <v>275.7312715228299</v>
       </c>
       <c r="P128" t="n">
-        <v>1799.945511522417</v>
+        <v>1799.945055930116</v>
       </c>
       <c r="Q128" t="n">
-        <v>156.4029358554356</v>
+        <v>156.4029162256924</v>
       </c>
       <c r="R128" t="n">
-        <v>835.847502367208</v>
+        <v>835.8475387962892</v>
       </c>
     </row>
     <row r="129">
@@ -7524,22 +7524,22 @@
         <v>3.39</v>
       </c>
       <c r="M129" t="n">
-        <v>209.85828338132</v>
+        <v>209.8583228113835</v>
       </c>
       <c r="N129" t="n">
-        <v>119.9050439428864</v>
+        <v>119.9050582521209</v>
       </c>
       <c r="O129" t="n">
-        <v>268.6691278766402</v>
+        <v>268.6691203236874</v>
       </c>
       <c r="P129" t="n">
-        <v>1821.889106651544</v>
+        <v>1821.888649998254</v>
       </c>
       <c r="Q129" t="n">
-        <v>164.7329364771359</v>
+        <v>164.7329281661491</v>
       </c>
       <c r="R129" t="n">
-        <v>789.2823709585531</v>
+        <v>789.2823511185147</v>
       </c>
     </row>
     <row r="130">
@@ -7580,22 +7580,22 @@
         <v>3.45</v>
       </c>
       <c r="M130" t="n">
-        <v>215.9361465504395</v>
+        <v>215.9361758666363</v>
       </c>
       <c r="N130" t="n">
-        <v>124.6630033779737</v>
+        <v>124.6630088256139</v>
       </c>
       <c r="O130" t="n">
-        <v>274.9330622738136</v>
+        <v>274.9330703013908</v>
       </c>
       <c r="P130" t="n">
-        <v>1799.197666288034</v>
+        <v>1799.197219063426</v>
       </c>
       <c r="Q130" t="n">
-        <v>168.8085553685743</v>
+        <v>168.8085473790997</v>
       </c>
       <c r="R130" t="n">
-        <v>812.6437049544469</v>
+        <v>812.6436963930518</v>
       </c>
     </row>
     <row r="131">
@@ -7636,22 +7636,22 @@
         <v>3.49</v>
       </c>
       <c r="M131" t="n">
-        <v>213.4748809127023</v>
+        <v>213.474917997469</v>
       </c>
       <c r="N131" t="n">
-        <v>126.3465107099351</v>
+        <v>126.3465214209182</v>
       </c>
       <c r="O131" t="n">
-        <v>273.1133072706958</v>
+        <v>273.1132950630014</v>
       </c>
       <c r="P131" t="n">
-        <v>2135.05680078673</v>
+        <v>2135.056270077982</v>
       </c>
       <c r="Q131" t="n">
-        <v>163.8540330287217</v>
+        <v>163.8540223071288</v>
       </c>
       <c r="R131" t="n">
-        <v>879.284278047472</v>
+        <v>879.2842891867359</v>
       </c>
     </row>
     <row r="132">
@@ -7692,22 +7692,22 @@
         <v>3.47</v>
       </c>
       <c r="M132" t="n">
-        <v>219.4232437165053</v>
+        <v>219.4232631842567</v>
       </c>
       <c r="N132" t="n">
-        <v>124.9059033755876</v>
+        <v>124.9059122730713</v>
       </c>
       <c r="O132" t="n">
-        <v>287.1094721487543</v>
+        <v>287.1094742512445</v>
       </c>
       <c r="P132" t="n">
-        <v>1935.453631916823</v>
+        <v>1935.453150823216</v>
       </c>
       <c r="Q132" t="n">
-        <v>141.2916699352634</v>
+        <v>141.2916555045615</v>
       </c>
       <c r="R132" t="n">
-        <v>883.6802952796814</v>
+        <v>883.6802751188811</v>
       </c>
     </row>
     <row r="133">
@@ -7748,22 +7748,22 @@
         <v>3.49</v>
       </c>
       <c r="M133" t="n">
-        <v>233.312436893341</v>
+        <v>233.3124641907131</v>
       </c>
       <c r="N133" t="n">
-        <v>128.7451874917095</v>
+        <v>128.7451974443491</v>
       </c>
       <c r="O133" t="n">
-        <v>287.6378085348784</v>
+        <v>287.6378025564842</v>
       </c>
       <c r="P133" t="n">
-        <v>1734.405043687135</v>
+        <v>1734.404612567958</v>
       </c>
       <c r="Q133" t="n">
-        <v>154.0389451310591</v>
+        <v>154.0389296063228</v>
       </c>
       <c r="R133" t="n">
-        <v>950.876095230484</v>
+        <v>950.8761459414382</v>
       </c>
     </row>
     <row r="134">
@@ -7804,22 +7804,22 @@
         <v>3.5</v>
       </c>
       <c r="M134" t="n">
-        <v>251.8752991114414</v>
+        <v>251.8753308285132</v>
       </c>
       <c r="N134" t="n">
-        <v>129.3130829328987</v>
+        <v>129.3130924097625</v>
       </c>
       <c r="O134" t="n">
-        <v>312.5393331490387</v>
+        <v>312.5393366071312</v>
       </c>
       <c r="P134" t="n">
-        <v>1715.302192576592</v>
+        <v>1715.301766205791</v>
       </c>
       <c r="Q134" t="n">
-        <v>152.0508567752879</v>
+        <v>152.0508417495114</v>
       </c>
       <c r="R134" t="n">
-        <v>953.7591106305374</v>
+        <v>953.7590967172964</v>
       </c>
     </row>
     <row r="135">
@@ -7860,22 +7860,22 @@
         <v>3.48</v>
       </c>
       <c r="M135" t="n">
-        <v>248.7708569527701</v>
+        <v>248.7708985027525</v>
       </c>
       <c r="N135" t="n">
-        <v>127.2490305146644</v>
+        <v>127.2490432555585</v>
       </c>
       <c r="O135" t="n">
-        <v>311.1048947977416</v>
+        <v>311.1049131208214</v>
       </c>
       <c r="P135" t="n">
-        <v>1665.420265930997</v>
+        <v>1665.419851959292</v>
       </c>
       <c r="Q135" t="n">
-        <v>149.3331412001643</v>
+        <v>149.3331386380426</v>
       </c>
       <c r="R135" t="n">
-        <v>904.2542902011654</v>
+        <v>904.2543113616899</v>
       </c>
     </row>
     <row r="136">
@@ -7916,22 +7916,22 @@
         <v>3.63</v>
       </c>
       <c r="M136" t="n">
-        <v>241.6999841774293</v>
+        <v>241.7000161782435</v>
       </c>
       <c r="N136" t="n">
-        <v>138.5071525678469</v>
+        <v>138.507165389852</v>
       </c>
       <c r="O136" t="n">
-        <v>297.925329919361</v>
+        <v>297.9253337631155</v>
       </c>
       <c r="P136" t="n">
-        <v>1571.707852694228</v>
+        <v>1571.707462016516</v>
       </c>
       <c r="Q136" t="n">
-        <v>194.0739006780349</v>
+        <v>194.0738908462248</v>
       </c>
       <c r="R136" t="n">
-        <v>1050.644362338325</v>
+        <v>1050.644365832527</v>
       </c>
     </row>
     <row r="137">
@@ -7972,22 +7972,22 @@
         <v>3.57</v>
       </c>
       <c r="M137" t="n">
-        <v>240.9318746218474</v>
+        <v>240.9319162519621</v>
       </c>
       <c r="N137" t="n">
-        <v>140.2206837943386</v>
+        <v>140.2206935106626</v>
       </c>
       <c r="O137" t="n">
-        <v>309.792298064396</v>
+        <v>309.7923022056781</v>
       </c>
       <c r="P137" t="n">
-        <v>2066.956584835947</v>
+        <v>2066.956071054796</v>
       </c>
       <c r="Q137" t="n">
-        <v>188.2776693281026</v>
+        <v>188.2776594987787</v>
       </c>
       <c r="R137" t="n">
-        <v>1126.118985555578</v>
+        <v>1126.119005653612</v>
       </c>
     </row>
     <row r="138">
@@ -8028,22 +8028,22 @@
         <v>3.56</v>
       </c>
       <c r="M138" t="n">
-        <v>236.440570318205</v>
+        <v>236.4405997065748</v>
       </c>
       <c r="N138" t="n">
-        <v>132.5133127312455</v>
+        <v>132.5133241060677</v>
       </c>
       <c r="O138" t="n">
-        <v>297.0923627608261</v>
+        <v>297.0923805111221</v>
       </c>
       <c r="P138" t="n">
-        <v>2483.469090058528</v>
+        <v>2483.468472745317</v>
       </c>
       <c r="Q138" t="n">
-        <v>171.3966890735434</v>
+        <v>171.3966804885411</v>
       </c>
       <c r="R138" t="n">
-        <v>1215.377150615032</v>
+        <v>1215.377236072726</v>
       </c>
     </row>
     <row r="139">
@@ -8084,22 +8084,22 @@
         <v>3.6</v>
       </c>
       <c r="M139" t="n">
-        <v>238.330815992489</v>
+        <v>238.3308489700074</v>
       </c>
       <c r="N139" t="n">
-        <v>138.2781574740749</v>
+        <v>138.2781703673502</v>
       </c>
       <c r="O139" t="n">
-        <v>296.0761817771554</v>
+        <v>296.0761892466926</v>
       </c>
       <c r="P139" t="n">
-        <v>2590.266321570622</v>
+        <v>2590.265677710939</v>
       </c>
       <c r="Q139" t="n">
-        <v>164.2862585537657</v>
+        <v>164.2862530981817</v>
       </c>
       <c r="R139" t="n">
-        <v>1039.542165363492</v>
+        <v>1039.542170052306</v>
       </c>
     </row>
     <row r="140">
@@ -8140,22 +8140,22 @@
         <v>3.7</v>
       </c>
       <c r="M140" t="n">
-        <v>250.4626357120475</v>
+        <v>250.4626743641255</v>
       </c>
       <c r="N140" t="n">
-        <v>145.2305260137706</v>
+        <v>145.2305370192541</v>
       </c>
       <c r="O140" t="n">
-        <v>294.3227108240779</v>
+        <v>294.3227180879117</v>
       </c>
       <c r="P140" t="n">
-        <v>2723.766231669023</v>
+        <v>2723.765554625413</v>
       </c>
       <c r="Q140" t="n">
-        <v>176.1758554572894</v>
+        <v>176.1758490651983</v>
       </c>
       <c r="R140" t="n">
-        <v>1043.998388252396</v>
+        <v>1043.998414082081</v>
       </c>
     </row>
     <row r="141">
@@ -8196,22 +8196,22 @@
         <v>3.8</v>
       </c>
       <c r="M141" t="n">
-        <v>247.4756116185166</v>
+        <v>247.4756467383139</v>
       </c>
       <c r="N141" t="n">
-        <v>152.1903958489648</v>
+        <v>152.1904059461645</v>
       </c>
       <c r="O141" t="n">
-        <v>297.6635464238987</v>
+        <v>297.6635574968354</v>
       </c>
       <c r="P141" t="n">
-        <v>2759.294657040779</v>
+        <v>2759.293971165907</v>
       </c>
       <c r="Q141" t="n">
-        <v>172.5598037154035</v>
+        <v>172.5597940841508</v>
       </c>
       <c r="R141" t="n">
-        <v>1039.975321119678</v>
+        <v>1039.975326309881</v>
       </c>
     </row>
   </sheetData>

</xml_diff>